<commit_message>
update unit8 to 12
</commit_message>
<xml_diff>
--- a/unit8_device_tree/Petazzoni-device-tree-dummies.xlsx
+++ b/unit8_device_tree/Petazzoni-device-tree-dummies.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Game\Linux\unit8_device_tree\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD27A1BC-60F9-4CC0-A90B-BE7DEEB2290C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B80AA65D-1514-4EE4-9B16-4310320A517C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{A56FE4C5-6830-46AE-AB8F-5BA0BAFCC647}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A56FE4C5-6830-46AE-AB8F-5BA0BAFCC647}"/>
   </bookViews>
   <sheets>
     <sheet name="MucLuc" sheetId="2" r:id="rId1"/>
@@ -5843,7 +5843,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -5925,6 +5925,88 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="11" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="13" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="12" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -5977,99 +6059,15 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="11" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="13" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="12" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -6914,142 +6912,116 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FEF9897-2408-4042-985C-A1698893C665}">
-  <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="B2:E12"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="96"/>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="96"/>
-      <c r="B2" s="98" t="s">
+    <row r="2" spans="2:5">
+      <c r="B2" s="78" t="s">
         <v>515</v>
       </c>
-      <c r="C2" s="99"/>
-      <c r="D2" s="99"/>
-      <c r="E2" s="100"/>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="96"/>
-      <c r="B3" s="97">
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="80"/>
+    </row>
+    <row r="3" spans="2:5">
+      <c r="B3" s="74">
         <v>1</v>
       </c>
-      <c r="C3" s="101" t="s">
+      <c r="C3" s="75" t="s">
         <v>523</v>
       </c>
-      <c r="D3" s="102"/>
-      <c r="E3" s="103"/>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="96"/>
-      <c r="B4" s="97">
+      <c r="D3" s="76"/>
+      <c r="E3" s="77"/>
+    </row>
+    <row r="4" spans="2:5">
+      <c r="B4" s="74">
         <v>2</v>
       </c>
-      <c r="C4" s="101" t="s">
+      <c r="C4" s="75" t="s">
         <v>524</v>
       </c>
-      <c r="D4" s="102"/>
-      <c r="E4" s="103"/>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="96"/>
-      <c r="B5" s="97">
+      <c r="D4" s="76"/>
+      <c r="E4" s="77"/>
+    </row>
+    <row r="5" spans="2:5">
+      <c r="B5" s="74">
         <v>3</v>
       </c>
-      <c r="C5" s="101" t="s">
+      <c r="C5" s="75" t="s">
         <v>525</v>
       </c>
-      <c r="D5" s="102"/>
-      <c r="E5" s="103"/>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="96"/>
-      <c r="B6" s="97">
+      <c r="D5" s="76"/>
+      <c r="E5" s="77"/>
+    </row>
+    <row r="6" spans="2:5">
+      <c r="B6" s="74">
         <v>4</v>
       </c>
-      <c r="C6" s="101" t="s">
+      <c r="C6" s="75" t="s">
         <v>516</v>
       </c>
-      <c r="D6" s="102"/>
-      <c r="E6" s="103"/>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="96"/>
-      <c r="B7" s="97">
+      <c r="D6" s="76"/>
+      <c r="E6" s="77"/>
+    </row>
+    <row r="7" spans="2:5">
+      <c r="B7" s="74">
         <v>5</v>
       </c>
-      <c r="C7" s="101" t="s">
+      <c r="C7" s="75" t="s">
         <v>517</v>
       </c>
-      <c r="D7" s="102"/>
-      <c r="E7" s="103"/>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8" s="96"/>
-      <c r="B8" s="97">
+      <c r="D7" s="76"/>
+      <c r="E7" s="77"/>
+    </row>
+    <row r="8" spans="2:5">
+      <c r="B8" s="74">
         <v>6</v>
       </c>
-      <c r="C8" s="101" t="s">
+      <c r="C8" s="75" t="s">
         <v>518</v>
       </c>
-      <c r="D8" s="102"/>
-      <c r="E8" s="103"/>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" s="96"/>
-      <c r="B9" s="97">
+      <c r="D8" s="76"/>
+      <c r="E8" s="77"/>
+    </row>
+    <row r="9" spans="2:5">
+      <c r="B9" s="74">
         <v>7</v>
       </c>
-      <c r="C9" s="101" t="s">
+      <c r="C9" s="75" t="s">
         <v>519</v>
       </c>
-      <c r="D9" s="102"/>
-      <c r="E9" s="103"/>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="96"/>
-      <c r="B10" s="97">
+      <c r="D9" s="76"/>
+      <c r="E9" s="77"/>
+    </row>
+    <row r="10" spans="2:5">
+      <c r="B10" s="74">
         <v>8</v>
       </c>
-      <c r="C10" s="101" t="s">
+      <c r="C10" s="75" t="s">
         <v>520</v>
       </c>
-      <c r="D10" s="102"/>
-      <c r="E10" s="103"/>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="96"/>
-      <c r="B11" s="97">
+      <c r="D10" s="76"/>
+      <c r="E10" s="77"/>
+    </row>
+    <row r="11" spans="2:5">
+      <c r="B11" s="74">
         <v>9</v>
       </c>
-      <c r="C11" s="101" t="s">
+      <c r="C11" s="75" t="s">
         <v>521</v>
       </c>
-      <c r="D11" s="102"/>
-      <c r="E11" s="103"/>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" s="96"/>
-      <c r="B12" s="97">
+      <c r="D11" s="76"/>
+      <c r="E11" s="77"/>
+    </row>
+    <row r="12" spans="2:5">
+      <c r="B12" s="74">
         <v>10</v>
       </c>
-      <c r="C12" s="101" t="s">
+      <c r="C12" s="75" t="s">
         <v>522</v>
       </c>
-      <c r="D12" s="102"/>
-      <c r="E12" s="103"/>
-      <c r="G12" s="62"/>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="A13" s="96"/>
-      <c r="B13" s="96"/>
-      <c r="C13" s="96"/>
-      <c r="D13" s="96"/>
-      <c r="E13" s="96"/>
+      <c r="D12" s="76"/>
+      <c r="E12" s="77"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -7058,12 +7030,12 @@
     <mergeCell ref="C10:E10"/>
     <mergeCell ref="C11:E11"/>
     <mergeCell ref="C12:E12"/>
+    <mergeCell ref="C7:E7"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="C4:E4"/>
     <mergeCell ref="C5:E5"/>
     <mergeCell ref="C6:E6"/>
-    <mergeCell ref="C7:E7"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B2" location="MucLuc!A1" display="MucLuc" xr:uid="{BF9E6673-44EB-427D-B554-0A4F98CE8903}"/>
@@ -7085,9 +7057,9 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C02540E6-78B8-4A3D-9DEC-8A52DC578F1E}">
   <dimension ref="B1:U89"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <sheetData>
-    <row r="1" spans="2:5" ht="23.25">
+    <row r="1" spans="2:5" ht="22.8">
       <c r="B1" s="1" t="s">
         <v>337</v>
       </c>
@@ -7122,12 +7094,12 @@
         <v>343</v>
       </c>
     </row>
-    <row r="8" spans="2:5" ht="23.25">
+    <row r="8" spans="2:5" ht="22.8">
       <c r="B8" s="1" t="s">
         <v>344</v>
       </c>
     </row>
-    <row r="9" spans="2:5" ht="17.25">
+    <row r="9" spans="2:5" ht="17.399999999999999">
       <c r="C9" s="2" t="s">
         <v>345</v>
       </c>
@@ -7147,7 +7119,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="13" spans="2:5" ht="15">
+    <row r="13" spans="2:5">
       <c r="C13" s="3"/>
       <c r="D13" s="8" t="s">
         <v>349</v>
@@ -7163,7 +7135,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="16" spans="2:5" ht="17.25">
+    <row r="16" spans="2:5" ht="17.399999999999999">
       <c r="C16" s="2" t="s">
         <v>352</v>
       </c>
@@ -7188,17 +7160,17 @@
         <v>356</v>
       </c>
     </row>
-    <row r="21" spans="2:21" ht="23.25">
+    <row r="21" spans="2:21" ht="22.8">
       <c r="B21" s="1" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="22" spans="2:21" ht="15">
+    <row r="22" spans="2:21">
       <c r="C22" s="8" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="23" spans="2:21" ht="15">
+    <row r="23" spans="2:21">
       <c r="C23" s="8" t="s">
         <v>359</v>
       </c>
@@ -7218,28 +7190,28 @@
         <v>362</v>
       </c>
     </row>
-    <row r="27" spans="2:21" ht="23.25">
+    <row r="27" spans="2:21" ht="22.8">
       <c r="B27" s="1" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="28" spans="2:21" ht="18">
-      <c r="B28" s="55" t="s">
+    <row r="28" spans="2:21" ht="17.399999999999999">
+      <c r="B28" s="37" t="s">
         <v>364</v>
       </c>
-      <c r="J28" s="56" t="s">
+      <c r="J28" s="38" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="29" spans="2:21" ht="18">
+    <row r="29" spans="2:21" ht="17.399999999999999">
       <c r="C29" s="4" t="s">
         <v>365</v>
       </c>
-      <c r="J29" s="56" t="s">
+      <c r="J29" s="38" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="30" spans="2:21" ht="23.25">
+    <row r="30" spans="2:21" ht="22.8">
       <c r="C30" s="4" t="s">
         <v>366</v>
       </c>
@@ -7247,127 +7219,127 @@
         <v>393</v>
       </c>
     </row>
-    <row r="31" spans="2:21" ht="15">
+    <row r="31" spans="2:21">
       <c r="C31" s="4" t="s">
         <v>367</v>
       </c>
-      <c r="K31" s="57" t="s">
+      <c r="K31" s="100" t="s">
         <v>394</v>
       </c>
-      <c r="L31" s="57"/>
-      <c r="M31" s="57" t="s">
+      <c r="L31" s="100"/>
+      <c r="M31" s="100" t="s">
         <v>186</v>
       </c>
-      <c r="N31" s="57"/>
-      <c r="O31" s="57"/>
-      <c r="P31" s="57"/>
-      <c r="Q31" s="57"/>
-      <c r="R31" s="57"/>
-      <c r="S31" s="57"/>
-      <c r="T31" s="57"/>
-      <c r="U31" s="57"/>
+      <c r="N31" s="100"/>
+      <c r="O31" s="100"/>
+      <c r="P31" s="100"/>
+      <c r="Q31" s="100"/>
+      <c r="R31" s="100"/>
+      <c r="S31" s="100"/>
+      <c r="T31" s="100"/>
+      <c r="U31" s="100"/>
     </row>
     <row r="32" spans="2:21">
       <c r="C32" s="4" t="s">
         <v>368</v>
       </c>
-      <c r="K32" s="58" t="s">
+      <c r="K32" s="99" t="s">
         <v>219</v>
       </c>
-      <c r="L32" s="58"/>
-      <c r="M32" s="59" t="s">
+      <c r="L32" s="99"/>
+      <c r="M32" s="101" t="s">
         <v>395</v>
       </c>
-      <c r="N32" s="59"/>
-      <c r="O32" s="59"/>
-      <c r="P32" s="59"/>
-      <c r="Q32" s="59"/>
-      <c r="R32" s="59"/>
-      <c r="S32" s="59"/>
-      <c r="T32" s="59"/>
-      <c r="U32" s="59"/>
+      <c r="N32" s="101"/>
+      <c r="O32" s="101"/>
+      <c r="P32" s="101"/>
+      <c r="Q32" s="101"/>
+      <c r="R32" s="101"/>
+      <c r="S32" s="101"/>
+      <c r="T32" s="101"/>
+      <c r="U32" s="101"/>
     </row>
     <row r="33" spans="2:21">
       <c r="C33" s="4" t="s">
         <v>369</v>
       </c>
-      <c r="K33" s="58" t="s">
+      <c r="K33" s="99" t="s">
         <v>396</v>
       </c>
-      <c r="L33" s="58"/>
-      <c r="M33" s="59" t="s">
+      <c r="L33" s="99"/>
+      <c r="M33" s="101" t="s">
         <v>397</v>
       </c>
-      <c r="N33" s="59"/>
-      <c r="O33" s="59"/>
-      <c r="P33" s="59"/>
-      <c r="Q33" s="59"/>
-      <c r="R33" s="59"/>
-      <c r="S33" s="59"/>
-      <c r="T33" s="59"/>
-      <c r="U33" s="59"/>
+      <c r="N33" s="101"/>
+      <c r="O33" s="101"/>
+      <c r="P33" s="101"/>
+      <c r="Q33" s="101"/>
+      <c r="R33" s="101"/>
+      <c r="S33" s="101"/>
+      <c r="T33" s="101"/>
+      <c r="U33" s="101"/>
     </row>
     <row r="34" spans="2:21" ht="29.25" customHeight="1">
       <c r="C34" s="4" t="s">
         <v>370</v>
       </c>
-      <c r="K34" s="58" t="s">
+      <c r="K34" s="99" t="s">
         <v>398</v>
       </c>
-      <c r="L34" s="58"/>
-      <c r="M34" s="59" t="s">
+      <c r="L34" s="99"/>
+      <c r="M34" s="101" t="s">
         <v>399</v>
       </c>
-      <c r="N34" s="59"/>
-      <c r="O34" s="59"/>
-      <c r="P34" s="59"/>
-      <c r="Q34" s="59"/>
-      <c r="R34" s="59"/>
-      <c r="S34" s="59"/>
-      <c r="T34" s="59"/>
-      <c r="U34" s="59"/>
+      <c r="N34" s="101"/>
+      <c r="O34" s="101"/>
+      <c r="P34" s="101"/>
+      <c r="Q34" s="101"/>
+      <c r="R34" s="101"/>
+      <c r="S34" s="101"/>
+      <c r="T34" s="101"/>
+      <c r="U34" s="101"/>
     </row>
     <row r="35" spans="2:21">
       <c r="C35" s="4" t="s">
         <v>371</v>
       </c>
-      <c r="K35" s="58" t="s">
+      <c r="K35" s="99" t="s">
         <v>400</v>
       </c>
-      <c r="L35" s="58"/>
-      <c r="M35" s="59" t="s">
+      <c r="L35" s="99"/>
+      <c r="M35" s="101" t="s">
         <v>401</v>
       </c>
-      <c r="N35" s="59"/>
-      <c r="O35" s="59"/>
-      <c r="P35" s="59"/>
-      <c r="Q35" s="59"/>
-      <c r="R35" s="59"/>
-      <c r="S35" s="59"/>
-      <c r="T35" s="59"/>
-      <c r="U35" s="59"/>
+      <c r="N35" s="101"/>
+      <c r="O35" s="101"/>
+      <c r="P35" s="101"/>
+      <c r="Q35" s="101"/>
+      <c r="R35" s="101"/>
+      <c r="S35" s="101"/>
+      <c r="T35" s="101"/>
+      <c r="U35" s="101"/>
     </row>
     <row r="36" spans="2:21">
       <c r="C36" s="4" t="s">
         <v>372</v>
       </c>
-      <c r="K36" s="58" t="s">
+      <c r="K36" s="99" t="s">
         <v>402</v>
       </c>
-      <c r="L36" s="58"/>
-      <c r="M36" s="59" t="s">
+      <c r="L36" s="99"/>
+      <c r="M36" s="101" t="s">
         <v>403</v>
       </c>
-      <c r="N36" s="59"/>
-      <c r="O36" s="59"/>
-      <c r="P36" s="59"/>
-      <c r="Q36" s="59"/>
-      <c r="R36" s="59"/>
-      <c r="S36" s="59"/>
-      <c r="T36" s="59"/>
-      <c r="U36" s="59"/>
-    </row>
-    <row r="37" spans="2:21" ht="23.25">
+      <c r="N36" s="101"/>
+      <c r="O36" s="101"/>
+      <c r="P36" s="101"/>
+      <c r="Q36" s="101"/>
+      <c r="R36" s="101"/>
+      <c r="S36" s="101"/>
+      <c r="T36" s="101"/>
+      <c r="U36" s="101"/>
+    </row>
+    <row r="37" spans="2:21" ht="22.8">
       <c r="C37" s="4" t="s">
         <v>373</v>
       </c>
@@ -7403,7 +7375,7 @@
       <c r="C41" s="4" t="s">
         <v>375</v>
       </c>
-      <c r="K41" s="51"/>
+      <c r="K41" s="33"/>
     </row>
     <row r="42" spans="2:21">
       <c r="C42" s="4" t="s">
@@ -7419,7 +7391,7 @@
       </c>
     </row>
     <row r="44" spans="2:21">
-      <c r="B44" s="55" t="s">
+      <c r="B44" s="37" t="s">
         <v>376</v>
       </c>
       <c r="K44" s="4" t="s">
@@ -7454,7 +7426,7 @@
       <c r="C48" s="4" t="s">
         <v>379</v>
       </c>
-      <c r="K48" s="51"/>
+      <c r="K48" s="33"/>
     </row>
     <row r="49" spans="3:11">
       <c r="C49" s="4" t="s">
@@ -7473,7 +7445,7 @@
       </c>
     </row>
     <row r="51" spans="3:11">
-      <c r="C51" s="51"/>
+      <c r="C51" s="33"/>
       <c r="K51" s="4" t="s">
         <v>413</v>
       </c>
@@ -7490,7 +7462,7 @@
       <c r="C53" s="4" t="s">
         <v>382</v>
       </c>
-      <c r="K53" s="51"/>
+      <c r="K53" s="33"/>
     </row>
     <row r="54" spans="3:11">
       <c r="C54" s="4" t="s">
@@ -7501,7 +7473,7 @@
       </c>
     </row>
     <row r="55" spans="3:11">
-      <c r="C55" s="51"/>
+      <c r="C55" s="33"/>
       <c r="K55" s="4" t="s">
         <v>295</v>
       </c>
@@ -7522,7 +7494,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="58" spans="3:11" ht="15">
+    <row r="58" spans="3:11">
       <c r="C58" s="4" t="s">
         <v>384</v>
       </c>
@@ -7536,13 +7508,13 @@
       </c>
       <c r="J59" s="3"/>
     </row>
-    <row r="60" spans="3:11" ht="23.25">
-      <c r="C60" s="51"/>
+    <row r="60" spans="3:11" ht="22.8">
+      <c r="C60" s="33"/>
       <c r="J60" s="1" t="s">
         <v>417</v>
       </c>
     </row>
-    <row r="61" spans="3:11" ht="15">
+    <row r="61" spans="3:11">
       <c r="C61" s="4" t="s">
         <v>385</v>
       </c>
@@ -7550,7 +7522,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="62" spans="3:11" ht="15">
+    <row r="62" spans="3:11">
       <c r="C62" s="4" t="s">
         <v>386</v>
       </c>
@@ -7558,7 +7530,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="63" spans="3:11" ht="15">
+    <row r="63" spans="3:11">
       <c r="C63" s="4" t="s">
         <v>387</v>
       </c>
@@ -7566,7 +7538,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="64" spans="3:11" ht="23.25">
+    <row r="64" spans="3:11" ht="22.8">
       <c r="C64" s="4" t="s">
         <v>388</v>
       </c>
@@ -7613,7 +7585,7 @@
       </c>
       <c r="J69" s="3"/>
     </row>
-    <row r="70" spans="2:11" ht="15">
+    <row r="70" spans="2:11">
       <c r="B70" s="3" t="s">
         <v>391</v>
       </c>
@@ -7627,25 +7599,25 @@
       </c>
       <c r="J71" s="3"/>
     </row>
-    <row r="75" spans="2:11" ht="17.25">
+    <row r="75" spans="2:11" ht="17.399999999999999">
       <c r="B75" s="2"/>
     </row>
     <row r="76" spans="2:11">
       <c r="B76" s="3"/>
     </row>
-    <row r="77" spans="2:11" ht="15">
+    <row r="77" spans="2:11">
       <c r="B77" s="8"/>
     </row>
     <row r="78" spans="2:11">
       <c r="B78" s="3"/>
     </row>
-    <row r="79" spans="2:11" ht="15">
+    <row r="79" spans="2:11">
       <c r="B79" s="8"/>
     </row>
     <row r="80" spans="2:11">
       <c r="B80" s="3"/>
     </row>
-    <row r="81" spans="2:2" ht="15">
+    <row r="81" spans="2:2">
       <c r="B81" s="8"/>
     </row>
     <row r="84" spans="2:2">
@@ -7668,11 +7640,6 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="K31:L31"/>
-    <mergeCell ref="K32:L32"/>
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="K34:L34"/>
-    <mergeCell ref="K35:L35"/>
     <mergeCell ref="K36:L36"/>
     <mergeCell ref="M31:U31"/>
     <mergeCell ref="M32:U32"/>
@@ -7680,6 +7647,11 @@
     <mergeCell ref="M34:U34"/>
     <mergeCell ref="M35:U35"/>
     <mergeCell ref="M36:U36"/>
+    <mergeCell ref="K31:L31"/>
+    <mergeCell ref="K32:L32"/>
+    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="K34:L34"/>
+    <mergeCell ref="K35:L35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7689,14 +7661,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FF50FC6-B31C-4E14-82D1-87AE5DBD189C}">
   <dimension ref="B2:O126"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <sheetData>
-    <row r="2" spans="2:3" ht="15">
+    <row r="2" spans="2:3">
       <c r="B2" s="9" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="3" spans="2:3" ht="15">
+    <row r="3" spans="2:3">
       <c r="B3" s="8" t="s">
         <v>430</v>
       </c>
@@ -7711,12 +7683,12 @@
         <v>432</v>
       </c>
     </row>
-    <row r="6" spans="2:3" ht="15">
+    <row r="6" spans="2:3">
       <c r="B6" s="8" t="s">
         <v>433</v>
       </c>
     </row>
-    <row r="7" spans="2:3" ht="15">
+    <row r="7" spans="2:3">
       <c r="B7" s="5" t="s">
         <v>434</v>
       </c>
@@ -7726,7 +7698,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="9" spans="2:3" ht="15">
+    <row r="9" spans="2:3">
       <c r="B9" s="8" t="s">
         <v>436</v>
       </c>
@@ -7784,19 +7756,19 @@
     <row r="20" spans="2:8">
       <c r="B20" s="3"/>
     </row>
-    <row r="21" spans="2:8" ht="15">
+    <row r="21" spans="2:8">
       <c r="B21" s="8" t="s">
         <v>447</v>
       </c>
     </row>
-    <row r="22" spans="2:8" ht="15">
+    <row r="22" spans="2:8">
       <c r="B22" s="3" t="s">
         <v>448</v>
       </c>
     </row>
     <row r="23" spans="2:8">
       <c r="B23" s="3"/>
-      <c r="C23" s="60" t="s">
+      <c r="C23" s="39" t="s">
         <v>449</v>
       </c>
       <c r="D23" s="17"/>
@@ -7806,157 +7778,97 @@
       <c r="H23" s="25"/>
     </row>
     <row r="24" spans="2:8">
-      <c r="C24" s="61" t="s">
+      <c r="C24" s="40" t="s">
         <v>450</v>
       </c>
-      <c r="D24" s="62"/>
-      <c r="E24" s="62"/>
-      <c r="F24" s="62"/>
-      <c r="G24" s="62"/>
       <c r="H24" s="27"/>
     </row>
     <row r="25" spans="2:8">
-      <c r="C25" s="61" t="s">
+      <c r="C25" s="40" t="s">
         <v>451</v>
       </c>
-      <c r="D25" s="62"/>
-      <c r="E25" s="62"/>
-      <c r="F25" s="62"/>
-      <c r="G25" s="62"/>
       <c r="H25" s="27"/>
     </row>
     <row r="26" spans="2:8">
-      <c r="C26" s="61" t="s">
+      <c r="C26" s="40" t="s">
         <v>452</v>
       </c>
-      <c r="D26" s="62"/>
-      <c r="E26" s="62"/>
-      <c r="F26" s="62"/>
-      <c r="G26" s="62"/>
       <c r="H26" s="27"/>
     </row>
     <row r="27" spans="2:8">
-      <c r="C27" s="61" t="s">
+      <c r="C27" s="40" t="s">
         <v>453</v>
       </c>
-      <c r="D27" s="62"/>
-      <c r="E27" s="62"/>
-      <c r="F27" s="62"/>
-      <c r="G27" s="62"/>
       <c r="H27" s="27"/>
     </row>
     <row r="28" spans="2:8">
-      <c r="C28" s="61" t="s">
+      <c r="C28" s="40" t="s">
         <v>454</v>
       </c>
-      <c r="D28" s="62"/>
-      <c r="E28" s="62"/>
-      <c r="F28" s="62"/>
-      <c r="G28" s="62"/>
       <c r="H28" s="27"/>
     </row>
     <row r="29" spans="2:8">
-      <c r="C29" s="61" t="s">
+      <c r="C29" s="40" t="s">
         <v>455</v>
       </c>
-      <c r="D29" s="62"/>
-      <c r="E29" s="62"/>
-      <c r="F29" s="62"/>
-      <c r="G29" s="62"/>
       <c r="H29" s="27"/>
     </row>
     <row r="30" spans="2:8">
-      <c r="C30" s="61" t="s">
+      <c r="C30" s="40" t="s">
         <v>456</v>
       </c>
-      <c r="D30" s="62"/>
-      <c r="E30" s="62"/>
-      <c r="F30" s="62"/>
-      <c r="G30" s="62"/>
       <c r="H30" s="27"/>
     </row>
     <row r="31" spans="2:8">
-      <c r="C31" s="61" t="s">
+      <c r="C31" s="40" t="s">
         <v>457</v>
       </c>
-      <c r="D31" s="62"/>
-      <c r="E31" s="62"/>
-      <c r="F31" s="62"/>
-      <c r="G31" s="62"/>
       <c r="H31" s="27"/>
     </row>
     <row r="32" spans="2:8">
-      <c r="C32" s="61" t="s">
+      <c r="C32" s="40" t="s">
         <v>458</v>
       </c>
-      <c r="D32" s="62"/>
-      <c r="E32" s="62"/>
-      <c r="F32" s="62"/>
-      <c r="G32" s="62"/>
       <c r="H32" s="27"/>
     </row>
     <row r="33" spans="2:8">
-      <c r="C33" s="61" t="s">
+      <c r="C33" s="40" t="s">
         <v>459</v>
       </c>
-      <c r="D33" s="62"/>
-      <c r="E33" s="62"/>
-      <c r="F33" s="62"/>
-      <c r="G33" s="62"/>
       <c r="H33" s="27"/>
     </row>
     <row r="34" spans="2:8">
-      <c r="C34" s="61" t="s">
+      <c r="C34" s="40" t="s">
         <v>460</v>
       </c>
-      <c r="D34" s="62"/>
-      <c r="E34" s="62"/>
-      <c r="F34" s="62"/>
-      <c r="G34" s="62"/>
       <c r="H34" s="27"/>
     </row>
     <row r="35" spans="2:8">
-      <c r="C35" s="61" t="s">
+      <c r="C35" s="40" t="s">
         <v>461</v>
       </c>
-      <c r="D35" s="62"/>
-      <c r="E35" s="62"/>
-      <c r="F35" s="62"/>
-      <c r="G35" s="62"/>
       <c r="H35" s="27"/>
     </row>
     <row r="36" spans="2:8">
-      <c r="C36" s="61" t="s">
+      <c r="C36" s="40" t="s">
         <v>462</v>
       </c>
-      <c r="D36" s="62"/>
-      <c r="E36" s="62"/>
-      <c r="F36" s="62"/>
-      <c r="G36" s="62"/>
       <c r="H36" s="27"/>
     </row>
     <row r="37" spans="2:8">
-      <c r="C37" s="61" t="s">
+      <c r="C37" s="40" t="s">
         <v>463</v>
       </c>
-      <c r="D37" s="62"/>
-      <c r="E37" s="62"/>
-      <c r="F37" s="62"/>
-      <c r="G37" s="62"/>
       <c r="H37" s="27"/>
     </row>
     <row r="38" spans="2:8">
-      <c r="C38" s="61" t="s">
+      <c r="C38" s="40" t="s">
         <v>464</v>
       </c>
-      <c r="D38" s="62"/>
-      <c r="E38" s="62"/>
-      <c r="F38" s="62"/>
-      <c r="G38" s="62"/>
       <c r="H38" s="27"/>
     </row>
     <row r="39" spans="2:8">
-      <c r="C39" s="63" t="s">
+      <c r="C39" s="41" t="s">
         <v>465</v>
       </c>
       <c r="D39" s="29"/>
@@ -7965,652 +7877,652 @@
       <c r="G39" s="29"/>
       <c r="H39" s="30"/>
     </row>
-    <row r="40" spans="2:8" ht="15">
+    <row r="40" spans="2:8">
       <c r="B40" s="8" t="s">
         <v>466</v>
       </c>
     </row>
-    <row r="41" spans="2:8" ht="15">
+    <row r="41" spans="2:8">
       <c r="C41" s="16" t="s">
         <v>467</v>
       </c>
     </row>
-    <row r="42" spans="2:8" ht="15">
+    <row r="42" spans="2:8">
       <c r="C42" s="16" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="43" spans="2:8" ht="15">
+    <row r="43" spans="2:8">
       <c r="C43" s="16" t="s">
         <v>469</v>
       </c>
     </row>
-    <row r="44" spans="2:8" ht="15">
+    <row r="44" spans="2:8">
       <c r="B44" s="8" t="s">
         <v>470</v>
       </c>
     </row>
-    <row r="45" spans="2:8" ht="15">
+    <row r="45" spans="2:8">
       <c r="C45" s="16" t="s">
         <v>471</v>
       </c>
     </row>
-    <row r="46" spans="2:8" ht="15">
+    <row r="46" spans="2:8">
       <c r="C46" s="16" t="s">
         <v>472</v>
       </c>
     </row>
-    <row r="47" spans="2:8" ht="15">
+    <row r="47" spans="2:8">
       <c r="C47" s="16" t="s">
         <v>473</v>
       </c>
     </row>
-    <row r="48" spans="2:8" ht="17.25">
+    <row r="48" spans="2:8" ht="17.399999999999999">
       <c r="B48" s="2" t="s">
         <v>474</v>
       </c>
     </row>
     <row r="49" spans="3:15">
-      <c r="C49" s="64" t="s">
+      <c r="C49" s="42" t="s">
         <v>475</v>
       </c>
-      <c r="D49" s="65"/>
-      <c r="E49" s="65"/>
-      <c r="F49" s="65"/>
-      <c r="G49" s="65"/>
-      <c r="H49" s="65"/>
-      <c r="I49" s="66"/>
-      <c r="K49" s="74" t="s">
+      <c r="D49" s="43"/>
+      <c r="E49" s="43"/>
+      <c r="F49" s="43"/>
+      <c r="G49" s="43"/>
+      <c r="H49" s="43"/>
+      <c r="I49" s="44"/>
+      <c r="K49" s="52" t="s">
         <v>500</v>
       </c>
-      <c r="L49" s="75"/>
-      <c r="M49" s="75"/>
-      <c r="N49" s="75"/>
-      <c r="O49" s="76"/>
+      <c r="L49" s="53"/>
+      <c r="M49" s="53"/>
+      <c r="N49" s="53"/>
+      <c r="O49" s="54"/>
     </row>
     <row r="50" spans="3:15">
-      <c r="C50" s="67" t="s">
+      <c r="C50" s="45" t="s">
         <v>476</v>
       </c>
-      <c r="D50" s="68"/>
-      <c r="E50" s="68"/>
-      <c r="F50" s="68"/>
-      <c r="G50" s="68"/>
-      <c r="H50" s="68"/>
-      <c r="I50" s="69"/>
-      <c r="K50" s="77"/>
-      <c r="L50" s="78" t="s">
+      <c r="D50" s="46"/>
+      <c r="E50" s="46"/>
+      <c r="F50" s="46"/>
+      <c r="G50" s="46"/>
+      <c r="H50" s="46"/>
+      <c r="I50" s="47"/>
+      <c r="K50" s="55"/>
+      <c r="L50" s="56" t="s">
         <v>501</v>
       </c>
-      <c r="M50" s="79"/>
-      <c r="N50" s="79"/>
-      <c r="O50" s="80"/>
+      <c r="M50" s="57"/>
+      <c r="N50" s="57"/>
+      <c r="O50" s="58"/>
     </row>
     <row r="51" spans="3:15">
-      <c r="C51" s="67" t="s">
+      <c r="C51" s="45" t="s">
         <v>477</v>
       </c>
-      <c r="D51" s="68"/>
-      <c r="E51" s="68"/>
-      <c r="F51" s="68"/>
-      <c r="G51" s="68"/>
-      <c r="H51" s="68"/>
-      <c r="I51" s="69"/>
-      <c r="K51" s="77"/>
-      <c r="L51" s="78" t="s">
+      <c r="D51" s="46"/>
+      <c r="E51" s="46"/>
+      <c r="F51" s="46"/>
+      <c r="G51" s="46"/>
+      <c r="H51" s="46"/>
+      <c r="I51" s="47"/>
+      <c r="K51" s="55"/>
+      <c r="L51" s="56" t="s">
         <v>502</v>
       </c>
-      <c r="M51" s="79"/>
-      <c r="N51" s="79"/>
-      <c r="O51" s="80"/>
+      <c r="M51" s="57"/>
+      <c r="N51" s="57"/>
+      <c r="O51" s="58"/>
     </row>
     <row r="52" spans="3:15">
-      <c r="C52" s="67" t="s">
+      <c r="C52" s="45" t="s">
         <v>478</v>
       </c>
-      <c r="D52" s="68"/>
-      <c r="E52" s="68"/>
-      <c r="F52" s="68"/>
-      <c r="G52" s="68"/>
-      <c r="H52" s="68"/>
-      <c r="I52" s="69"/>
-      <c r="K52" s="77"/>
-      <c r="L52" s="78" t="s">
+      <c r="D52" s="46"/>
+      <c r="E52" s="46"/>
+      <c r="F52" s="46"/>
+      <c r="G52" s="46"/>
+      <c r="H52" s="46"/>
+      <c r="I52" s="47"/>
+      <c r="K52" s="55"/>
+      <c r="L52" s="56" t="s">
         <v>503</v>
       </c>
-      <c r="M52" s="79"/>
-      <c r="N52" s="79"/>
-      <c r="O52" s="80"/>
+      <c r="M52" s="57"/>
+      <c r="N52" s="57"/>
+      <c r="O52" s="58"/>
     </row>
     <row r="53" spans="3:15">
-      <c r="C53" s="67" t="s">
+      <c r="C53" s="45" t="s">
         <v>479</v>
       </c>
-      <c r="D53" s="68"/>
-      <c r="E53" s="68"/>
-      <c r="F53" s="68"/>
-      <c r="G53" s="68"/>
-      <c r="H53" s="68"/>
-      <c r="I53" s="69"/>
-      <c r="K53" s="77"/>
-      <c r="L53" s="78" t="s">
+      <c r="D53" s="46"/>
+      <c r="E53" s="46"/>
+      <c r="F53" s="46"/>
+      <c r="G53" s="46"/>
+      <c r="H53" s="46"/>
+      <c r="I53" s="47"/>
+      <c r="K53" s="55"/>
+      <c r="L53" s="56" t="s">
         <v>504</v>
       </c>
-      <c r="M53" s="79"/>
-      <c r="N53" s="79"/>
-      <c r="O53" s="80"/>
+      <c r="M53" s="57"/>
+      <c r="N53" s="57"/>
+      <c r="O53" s="58"/>
     </row>
     <row r="54" spans="3:15">
-      <c r="C54" s="67" t="s">
+      <c r="C54" s="45" t="s">
         <v>480</v>
       </c>
-      <c r="D54" s="68"/>
-      <c r="E54" s="68"/>
-      <c r="F54" s="68"/>
-      <c r="G54" s="68"/>
-      <c r="H54" s="68"/>
-      <c r="I54" s="69"/>
-      <c r="K54" s="77"/>
-      <c r="L54" s="78" t="s">
+      <c r="D54" s="46"/>
+      <c r="E54" s="46"/>
+      <c r="F54" s="46"/>
+      <c r="G54" s="46"/>
+      <c r="H54" s="46"/>
+      <c r="I54" s="47"/>
+      <c r="K54" s="55"/>
+      <c r="L54" s="56" t="s">
         <v>505</v>
       </c>
-      <c r="M54" s="79"/>
-      <c r="N54" s="79"/>
-      <c r="O54" s="80"/>
+      <c r="M54" s="57"/>
+      <c r="N54" s="57"/>
+      <c r="O54" s="58"/>
     </row>
     <row r="55" spans="3:15">
-      <c r="C55" s="70"/>
-      <c r="D55" s="68"/>
-      <c r="E55" s="68"/>
-      <c r="F55" s="68"/>
-      <c r="G55" s="68"/>
-      <c r="H55" s="68"/>
-      <c r="I55" s="69"/>
-      <c r="K55" s="81"/>
-      <c r="L55" s="82" t="s">
+      <c r="C55" s="48"/>
+      <c r="D55" s="46"/>
+      <c r="E55" s="46"/>
+      <c r="F55" s="46"/>
+      <c r="G55" s="46"/>
+      <c r="H55" s="46"/>
+      <c r="I55" s="47"/>
+      <c r="K55" s="59"/>
+      <c r="L55" s="60" t="s">
         <v>295</v>
       </c>
-      <c r="M55" s="83"/>
-      <c r="N55" s="83"/>
-      <c r="O55" s="84"/>
+      <c r="M55" s="61"/>
+      <c r="N55" s="61"/>
+      <c r="O55" s="62"/>
     </row>
     <row r="56" spans="3:15">
-      <c r="C56" s="67" t="s">
+      <c r="C56" s="45" t="s">
         <v>455</v>
       </c>
-      <c r="D56" s="68"/>
-      <c r="E56" s="68"/>
-      <c r="F56" s="68"/>
-      <c r="G56" s="68"/>
-      <c r="H56" s="68"/>
-      <c r="I56" s="69"/>
+      <c r="D56" s="46"/>
+      <c r="E56" s="46"/>
+      <c r="F56" s="46"/>
+      <c r="G56" s="46"/>
+      <c r="H56" s="46"/>
+      <c r="I56" s="47"/>
     </row>
     <row r="57" spans="3:15">
-      <c r="C57" s="67" t="s">
+      <c r="C57" s="45" t="s">
         <v>456</v>
       </c>
-      <c r="D57" s="68"/>
-      <c r="E57" s="68"/>
-      <c r="F57" s="68"/>
-      <c r="G57" s="68"/>
-      <c r="H57" s="68"/>
-      <c r="I57" s="69"/>
+      <c r="D57" s="46"/>
+      <c r="E57" s="46"/>
+      <c r="F57" s="46"/>
+      <c r="G57" s="46"/>
+      <c r="H57" s="46"/>
+      <c r="I57" s="47"/>
     </row>
     <row r="58" spans="3:15">
-      <c r="C58" s="67" t="s">
+      <c r="C58" s="45" t="s">
         <v>481</v>
       </c>
-      <c r="D58" s="68"/>
-      <c r="E58" s="68"/>
-      <c r="F58" s="68"/>
-      <c r="G58" s="68"/>
-      <c r="H58" s="68"/>
-      <c r="I58" s="69"/>
-      <c r="K58" s="85" t="s">
+      <c r="D58" s="46"/>
+      <c r="E58" s="46"/>
+      <c r="F58" s="46"/>
+      <c r="G58" s="46"/>
+      <c r="H58" s="46"/>
+      <c r="I58" s="47"/>
+      <c r="K58" s="63" t="s">
         <v>506</v>
       </c>
-      <c r="L58" s="86"/>
-      <c r="M58" s="86"/>
-      <c r="N58" s="86"/>
-      <c r="O58" s="87"/>
+      <c r="L58" s="64"/>
+      <c r="M58" s="64"/>
+      <c r="N58" s="64"/>
+      <c r="O58" s="65"/>
     </row>
     <row r="59" spans="3:15">
-      <c r="C59" s="67" t="s">
+      <c r="C59" s="45" t="s">
         <v>457</v>
       </c>
-      <c r="D59" s="68"/>
-      <c r="E59" s="68"/>
-      <c r="F59" s="68"/>
-      <c r="G59" s="68"/>
-      <c r="H59" s="68"/>
-      <c r="I59" s="69"/>
-      <c r="K59" s="88"/>
-      <c r="L59" s="89"/>
-      <c r="M59" s="89"/>
-      <c r="N59" s="89"/>
-      <c r="O59" s="90"/>
+      <c r="D59" s="46"/>
+      <c r="E59" s="46"/>
+      <c r="F59" s="46"/>
+      <c r="G59" s="46"/>
+      <c r="H59" s="46"/>
+      <c r="I59" s="47"/>
+      <c r="K59" s="66"/>
+      <c r="L59" s="67"/>
+      <c r="M59" s="67"/>
+      <c r="N59" s="67"/>
+      <c r="O59" s="68"/>
     </row>
     <row r="60" spans="3:15">
-      <c r="C60" s="67" t="s">
+      <c r="C60" s="45" t="s">
         <v>482</v>
       </c>
-      <c r="D60" s="68"/>
-      <c r="E60" s="68"/>
-      <c r="F60" s="68"/>
-      <c r="G60" s="68"/>
-      <c r="H60" s="68"/>
-      <c r="I60" s="69"/>
-      <c r="K60" s="91" t="s">
+      <c r="D60" s="46"/>
+      <c r="E60" s="46"/>
+      <c r="F60" s="46"/>
+      <c r="G60" s="46"/>
+      <c r="H60" s="46"/>
+      <c r="I60" s="47"/>
+      <c r="K60" s="69" t="s">
         <v>507</v>
       </c>
-      <c r="L60" s="89"/>
-      <c r="M60" s="89"/>
-      <c r="N60" s="89"/>
-      <c r="O60" s="90"/>
+      <c r="L60" s="67"/>
+      <c r="M60" s="67"/>
+      <c r="N60" s="67"/>
+      <c r="O60" s="68"/>
     </row>
     <row r="61" spans="3:15">
-      <c r="C61" s="70"/>
-      <c r="D61" s="68"/>
-      <c r="E61" s="68"/>
-      <c r="F61" s="68"/>
-      <c r="G61" s="68"/>
-      <c r="H61" s="68"/>
-      <c r="I61" s="69"/>
-      <c r="K61" s="91" t="s">
+      <c r="C61" s="48"/>
+      <c r="D61" s="46"/>
+      <c r="E61" s="46"/>
+      <c r="F61" s="46"/>
+      <c r="G61" s="46"/>
+      <c r="H61" s="46"/>
+      <c r="I61" s="47"/>
+      <c r="K61" s="69" t="s">
         <v>508</v>
       </c>
-      <c r="L61" s="89"/>
-      <c r="M61" s="89"/>
-      <c r="N61" s="89"/>
-      <c r="O61" s="90"/>
+      <c r="L61" s="67"/>
+      <c r="M61" s="67"/>
+      <c r="N61" s="67"/>
+      <c r="O61" s="68"/>
     </row>
     <row r="62" spans="3:15">
-      <c r="C62" s="67" t="s">
+      <c r="C62" s="45" t="s">
         <v>483</v>
       </c>
-      <c r="D62" s="68"/>
-      <c r="E62" s="68"/>
-      <c r="F62" s="68"/>
-      <c r="G62" s="68"/>
-      <c r="H62" s="68"/>
-      <c r="I62" s="69"/>
-      <c r="K62" s="91" t="s">
+      <c r="D62" s="46"/>
+      <c r="E62" s="46"/>
+      <c r="F62" s="46"/>
+      <c r="G62" s="46"/>
+      <c r="H62" s="46"/>
+      <c r="I62" s="47"/>
+      <c r="K62" s="69" t="s">
         <v>509</v>
       </c>
-      <c r="L62" s="89"/>
-      <c r="M62" s="89"/>
-      <c r="N62" s="89"/>
-      <c r="O62" s="90"/>
+      <c r="L62" s="67"/>
+      <c r="M62" s="67"/>
+      <c r="N62" s="67"/>
+      <c r="O62" s="68"/>
     </row>
     <row r="63" spans="3:15">
-      <c r="C63" s="67" t="s">
+      <c r="C63" s="45" t="s">
         <v>484</v>
       </c>
-      <c r="D63" s="68"/>
-      <c r="E63" s="68"/>
-      <c r="F63" s="68"/>
-      <c r="G63" s="68"/>
-      <c r="H63" s="68"/>
-      <c r="I63" s="69"/>
-      <c r="K63" s="91" t="s">
+      <c r="D63" s="46"/>
+      <c r="E63" s="46"/>
+      <c r="F63" s="46"/>
+      <c r="G63" s="46"/>
+      <c r="H63" s="46"/>
+      <c r="I63" s="47"/>
+      <c r="K63" s="69" t="s">
         <v>295</v>
       </c>
-      <c r="L63" s="89"/>
-      <c r="M63" s="89"/>
-      <c r="N63" s="89"/>
-      <c r="O63" s="90"/>
+      <c r="L63" s="67"/>
+      <c r="M63" s="67"/>
+      <c r="N63" s="67"/>
+      <c r="O63" s="68"/>
     </row>
     <row r="64" spans="3:15">
-      <c r="C64" s="67" t="s">
+      <c r="C64" s="45" t="s">
         <v>485</v>
       </c>
-      <c r="D64" s="68"/>
-      <c r="E64" s="68"/>
-      <c r="F64" s="68"/>
-      <c r="G64" s="68"/>
-      <c r="H64" s="68"/>
-      <c r="I64" s="69"/>
-      <c r="K64" s="91" t="s">
+      <c r="D64" s="46"/>
+      <c r="E64" s="46"/>
+      <c r="F64" s="46"/>
+      <c r="G64" s="46"/>
+      <c r="H64" s="46"/>
+      <c r="I64" s="47"/>
+      <c r="K64" s="69" t="s">
         <v>510</v>
       </c>
-      <c r="L64" s="89"/>
-      <c r="M64" s="89"/>
-      <c r="N64" s="89"/>
-      <c r="O64" s="90"/>
+      <c r="L64" s="67"/>
+      <c r="M64" s="67"/>
+      <c r="N64" s="67"/>
+      <c r="O64" s="68"/>
     </row>
     <row r="65" spans="3:15">
-      <c r="C65" s="67" t="s">
+      <c r="C65" s="45" t="s">
         <v>486</v>
       </c>
-      <c r="D65" s="68"/>
-      <c r="E65" s="68"/>
-      <c r="F65" s="68"/>
-      <c r="G65" s="68"/>
-      <c r="H65" s="68"/>
-      <c r="I65" s="69"/>
-      <c r="K65" s="92"/>
-      <c r="L65" s="89"/>
-      <c r="M65" s="89"/>
-      <c r="N65" s="89"/>
-      <c r="O65" s="90"/>
+      <c r="D65" s="46"/>
+      <c r="E65" s="46"/>
+      <c r="F65" s="46"/>
+      <c r="G65" s="46"/>
+      <c r="H65" s="46"/>
+      <c r="I65" s="47"/>
+      <c r="K65" s="70"/>
+      <c r="L65" s="67"/>
+      <c r="M65" s="67"/>
+      <c r="N65" s="67"/>
+      <c r="O65" s="68"/>
     </row>
     <row r="66" spans="3:15">
-      <c r="C66" s="67" t="s">
+      <c r="C66" s="45" t="s">
         <v>487</v>
       </c>
-      <c r="D66" s="68"/>
-      <c r="E66" s="68"/>
-      <c r="F66" s="68"/>
-      <c r="G66" s="68"/>
-      <c r="H66" s="68"/>
-      <c r="I66" s="69"/>
-      <c r="K66" s="91" t="s">
+      <c r="D66" s="46"/>
+      <c r="E66" s="46"/>
+      <c r="F66" s="46"/>
+      <c r="G66" s="46"/>
+      <c r="H66" s="46"/>
+      <c r="I66" s="47"/>
+      <c r="K66" s="69" t="s">
         <v>511</v>
       </c>
-      <c r="L66" s="89"/>
-      <c r="M66" s="89"/>
-      <c r="N66" s="89"/>
-      <c r="O66" s="90"/>
+      <c r="L66" s="67"/>
+      <c r="M66" s="67"/>
+      <c r="N66" s="67"/>
+      <c r="O66" s="68"/>
     </row>
     <row r="67" spans="3:15">
-      <c r="C67" s="67" t="s">
+      <c r="C67" s="45" t="s">
         <v>487</v>
       </c>
-      <c r="D67" s="68"/>
-      <c r="E67" s="68"/>
-      <c r="F67" s="68"/>
-      <c r="G67" s="68"/>
-      <c r="H67" s="68"/>
-      <c r="I67" s="69"/>
-      <c r="K67" s="91" t="s">
+      <c r="D67" s="46"/>
+      <c r="E67" s="46"/>
+      <c r="F67" s="46"/>
+      <c r="G67" s="46"/>
+      <c r="H67" s="46"/>
+      <c r="I67" s="47"/>
+      <c r="K67" s="69" t="s">
         <v>324</v>
       </c>
-      <c r="L67" s="89"/>
-      <c r="M67" s="89"/>
-      <c r="N67" s="89"/>
-      <c r="O67" s="90"/>
+      <c r="L67" s="67"/>
+      <c r="M67" s="67"/>
+      <c r="N67" s="67"/>
+      <c r="O67" s="68"/>
     </row>
     <row r="68" spans="3:15">
-      <c r="C68" s="67" t="s">
+      <c r="C68" s="45" t="s">
         <v>488</v>
       </c>
-      <c r="D68" s="68"/>
-      <c r="E68" s="68"/>
-      <c r="F68" s="68"/>
-      <c r="G68" s="68"/>
-      <c r="H68" s="68"/>
-      <c r="I68" s="69"/>
-      <c r="K68" s="91" t="s">
+      <c r="D68" s="46"/>
+      <c r="E68" s="46"/>
+      <c r="F68" s="46"/>
+      <c r="G68" s="46"/>
+      <c r="H68" s="46"/>
+      <c r="I68" s="47"/>
+      <c r="K68" s="69" t="s">
         <v>296</v>
       </c>
-      <c r="L68" s="89"/>
-      <c r="M68" s="89"/>
-      <c r="N68" s="89"/>
-      <c r="O68" s="90"/>
+      <c r="L68" s="67"/>
+      <c r="M68" s="67"/>
+      <c r="N68" s="67"/>
+      <c r="O68" s="68"/>
     </row>
     <row r="69" spans="3:15">
-      <c r="C69" s="67" t="s">
+      <c r="C69" s="45" t="s">
         <v>489</v>
       </c>
-      <c r="D69" s="68"/>
-      <c r="E69" s="68"/>
-      <c r="F69" s="68"/>
-      <c r="G69" s="68"/>
-      <c r="H69" s="68"/>
-      <c r="I69" s="69"/>
-      <c r="K69" s="91" t="s">
+      <c r="D69" s="46"/>
+      <c r="E69" s="46"/>
+      <c r="F69" s="46"/>
+      <c r="G69" s="46"/>
+      <c r="H69" s="46"/>
+      <c r="I69" s="47"/>
+      <c r="K69" s="69" t="s">
         <v>326</v>
       </c>
-      <c r="L69" s="89"/>
-      <c r="M69" s="89"/>
-      <c r="N69" s="89"/>
-      <c r="O69" s="90"/>
+      <c r="L69" s="67"/>
+      <c r="M69" s="67"/>
+      <c r="N69" s="67"/>
+      <c r="O69" s="68"/>
     </row>
     <row r="70" spans="3:15">
-      <c r="C70" s="70"/>
-      <c r="D70" s="68"/>
-      <c r="E70" s="68"/>
-      <c r="F70" s="68"/>
-      <c r="G70" s="68"/>
-      <c r="H70" s="68"/>
-      <c r="I70" s="69"/>
-      <c r="K70" s="91" t="s">
+      <c r="C70" s="48"/>
+      <c r="D70" s="46"/>
+      <c r="E70" s="46"/>
+      <c r="F70" s="46"/>
+      <c r="G70" s="46"/>
+      <c r="H70" s="46"/>
+      <c r="I70" s="47"/>
+      <c r="K70" s="69" t="s">
         <v>512</v>
       </c>
-      <c r="L70" s="89"/>
-      <c r="M70" s="89"/>
-      <c r="N70" s="89"/>
-      <c r="O70" s="90"/>
+      <c r="L70" s="67"/>
+      <c r="M70" s="67"/>
+      <c r="N70" s="67"/>
+      <c r="O70" s="68"/>
     </row>
     <row r="71" spans="3:15">
-      <c r="C71" s="67" t="s">
+      <c r="C71" s="45" t="s">
         <v>490</v>
       </c>
-      <c r="D71" s="68"/>
-      <c r="E71" s="68"/>
-      <c r="F71" s="68"/>
-      <c r="G71" s="68"/>
-      <c r="H71" s="68"/>
-      <c r="I71" s="69"/>
-      <c r="K71" s="92"/>
-      <c r="L71" s="89"/>
-      <c r="M71" s="89"/>
-      <c r="N71" s="89"/>
-      <c r="O71" s="90"/>
+      <c r="D71" s="46"/>
+      <c r="E71" s="46"/>
+      <c r="F71" s="46"/>
+      <c r="G71" s="46"/>
+      <c r="H71" s="46"/>
+      <c r="I71" s="47"/>
+      <c r="K71" s="70"/>
+      <c r="L71" s="67"/>
+      <c r="M71" s="67"/>
+      <c r="N71" s="67"/>
+      <c r="O71" s="68"/>
     </row>
     <row r="72" spans="3:15">
-      <c r="C72" s="67" t="s">
+      <c r="C72" s="45" t="s">
         <v>491</v>
       </c>
-      <c r="D72" s="68"/>
-      <c r="E72" s="68"/>
-      <c r="F72" s="68"/>
-      <c r="G72" s="68"/>
-      <c r="H72" s="68"/>
-      <c r="I72" s="69"/>
-      <c r="K72" s="91" t="s">
+      <c r="D72" s="46"/>
+      <c r="E72" s="46"/>
+      <c r="F72" s="46"/>
+      <c r="G72" s="46"/>
+      <c r="H72" s="46"/>
+      <c r="I72" s="47"/>
+      <c r="K72" s="69" t="s">
         <v>333</v>
       </c>
-      <c r="L72" s="89"/>
-      <c r="M72" s="89"/>
-      <c r="N72" s="89"/>
-      <c r="O72" s="90"/>
+      <c r="L72" s="67"/>
+      <c r="M72" s="67"/>
+      <c r="N72" s="67"/>
+      <c r="O72" s="68"/>
     </row>
     <row r="73" spans="3:15">
-      <c r="C73" s="67" t="s">
+      <c r="C73" s="45" t="s">
         <v>485</v>
       </c>
-      <c r="D73" s="68"/>
-      <c r="E73" s="68"/>
-      <c r="F73" s="68"/>
-      <c r="G73" s="68"/>
-      <c r="H73" s="68"/>
-      <c r="I73" s="69"/>
-      <c r="K73" s="91" t="s">
+      <c r="D73" s="46"/>
+      <c r="E73" s="46"/>
+      <c r="F73" s="46"/>
+      <c r="G73" s="46"/>
+      <c r="H73" s="46"/>
+      <c r="I73" s="47"/>
+      <c r="K73" s="69" t="s">
         <v>297</v>
       </c>
-      <c r="L73" s="89"/>
-      <c r="M73" s="89"/>
-      <c r="N73" s="89"/>
-      <c r="O73" s="90"/>
+      <c r="L73" s="67"/>
+      <c r="M73" s="67"/>
+      <c r="N73" s="67"/>
+      <c r="O73" s="68"/>
     </row>
     <row r="74" spans="3:15">
-      <c r="C74" s="67" t="s">
+      <c r="C74" s="45" t="s">
         <v>486</v>
       </c>
-      <c r="D74" s="68"/>
-      <c r="E74" s="68"/>
-      <c r="F74" s="68"/>
-      <c r="G74" s="68"/>
-      <c r="H74" s="68"/>
-      <c r="I74" s="69"/>
-      <c r="K74" s="91" t="s">
+      <c r="D74" s="46"/>
+      <c r="E74" s="46"/>
+      <c r="F74" s="46"/>
+      <c r="G74" s="46"/>
+      <c r="H74" s="46"/>
+      <c r="I74" s="47"/>
+      <c r="K74" s="69" t="s">
         <v>513</v>
       </c>
-      <c r="L74" s="89"/>
-      <c r="M74" s="89"/>
-      <c r="N74" s="89"/>
-      <c r="O74" s="90"/>
+      <c r="L74" s="67"/>
+      <c r="M74" s="67"/>
+      <c r="N74" s="67"/>
+      <c r="O74" s="68"/>
     </row>
     <row r="75" spans="3:15">
-      <c r="C75" s="67" t="s">
+      <c r="C75" s="45" t="s">
         <v>487</v>
       </c>
-      <c r="D75" s="68"/>
-      <c r="E75" s="68"/>
-      <c r="F75" s="68"/>
-      <c r="G75" s="68"/>
-      <c r="H75" s="68"/>
-      <c r="I75" s="69"/>
-      <c r="K75" s="92"/>
-      <c r="L75" s="89"/>
-      <c r="M75" s="89"/>
-      <c r="N75" s="89"/>
-      <c r="O75" s="90"/>
+      <c r="D75" s="46"/>
+      <c r="E75" s="46"/>
+      <c r="F75" s="46"/>
+      <c r="G75" s="46"/>
+      <c r="H75" s="46"/>
+      <c r="I75" s="47"/>
+      <c r="K75" s="70"/>
+      <c r="L75" s="67"/>
+      <c r="M75" s="67"/>
+      <c r="N75" s="67"/>
+      <c r="O75" s="68"/>
     </row>
     <row r="76" spans="3:15">
-      <c r="C76" s="67" t="s">
+      <c r="C76" s="45" t="s">
         <v>492</v>
       </c>
-      <c r="D76" s="68"/>
-      <c r="E76" s="68"/>
-      <c r="F76" s="68"/>
-      <c r="G76" s="68"/>
-      <c r="H76" s="68"/>
-      <c r="I76" s="69"/>
-      <c r="K76" s="91" t="s">
+      <c r="D76" s="46"/>
+      <c r="E76" s="46"/>
+      <c r="F76" s="46"/>
+      <c r="G76" s="46"/>
+      <c r="H76" s="46"/>
+      <c r="I76" s="47"/>
+      <c r="K76" s="69" t="s">
         <v>514</v>
       </c>
-      <c r="L76" s="89"/>
-      <c r="M76" s="89"/>
-      <c r="N76" s="89"/>
-      <c r="O76" s="90"/>
+      <c r="L76" s="67"/>
+      <c r="M76" s="67"/>
+      <c r="N76" s="67"/>
+      <c r="O76" s="68"/>
     </row>
     <row r="77" spans="3:15">
-      <c r="C77" s="70"/>
-      <c r="D77" s="68"/>
-      <c r="E77" s="68"/>
-      <c r="F77" s="68"/>
-      <c r="G77" s="68"/>
-      <c r="H77" s="68"/>
-      <c r="I77" s="69"/>
-      <c r="K77" s="93" t="s">
+      <c r="C77" s="48"/>
+      <c r="D77" s="46"/>
+      <c r="E77" s="46"/>
+      <c r="F77" s="46"/>
+      <c r="G77" s="46"/>
+      <c r="H77" s="46"/>
+      <c r="I77" s="47"/>
+      <c r="K77" s="71" t="s">
         <v>298</v>
       </c>
-      <c r="L77" s="94"/>
-      <c r="M77" s="94"/>
-      <c r="N77" s="94"/>
-      <c r="O77" s="95"/>
+      <c r="L77" s="72"/>
+      <c r="M77" s="72"/>
+      <c r="N77" s="72"/>
+      <c r="O77" s="73"/>
     </row>
     <row r="78" spans="3:15">
-      <c r="C78" s="67" t="s">
+      <c r="C78" s="45" t="s">
         <v>493</v>
       </c>
-      <c r="D78" s="68"/>
-      <c r="E78" s="68"/>
-      <c r="F78" s="68"/>
-      <c r="G78" s="68"/>
-      <c r="H78" s="68"/>
-      <c r="I78" s="69"/>
+      <c r="D78" s="46"/>
+      <c r="E78" s="46"/>
+      <c r="F78" s="46"/>
+      <c r="G78" s="46"/>
+      <c r="H78" s="46"/>
+      <c r="I78" s="47"/>
     </row>
     <row r="79" spans="3:15">
-      <c r="C79" s="67" t="s">
+      <c r="C79" s="45" t="s">
         <v>494</v>
       </c>
-      <c r="D79" s="68"/>
-      <c r="E79" s="68"/>
-      <c r="F79" s="68"/>
-      <c r="G79" s="68"/>
-      <c r="H79" s="68"/>
-      <c r="I79" s="69"/>
+      <c r="D79" s="46"/>
+      <c r="E79" s="46"/>
+      <c r="F79" s="46"/>
+      <c r="G79" s="46"/>
+      <c r="H79" s="46"/>
+      <c r="I79" s="47"/>
     </row>
     <row r="80" spans="3:15">
-      <c r="C80" s="67" t="s">
+      <c r="C80" s="45" t="s">
         <v>495</v>
       </c>
-      <c r="D80" s="68"/>
-      <c r="E80" s="68"/>
-      <c r="F80" s="68"/>
-      <c r="G80" s="68"/>
-      <c r="H80" s="68"/>
-      <c r="I80" s="69"/>
+      <c r="D80" s="46"/>
+      <c r="E80" s="46"/>
+      <c r="F80" s="46"/>
+      <c r="G80" s="46"/>
+      <c r="H80" s="46"/>
+      <c r="I80" s="47"/>
     </row>
     <row r="81" spans="3:9">
-      <c r="C81" s="67" t="s">
+      <c r="C81" s="45" t="s">
         <v>496</v>
       </c>
-      <c r="D81" s="68"/>
-      <c r="E81" s="68"/>
-      <c r="F81" s="68"/>
-      <c r="G81" s="68"/>
-      <c r="H81" s="68"/>
-      <c r="I81" s="69"/>
+      <c r="D81" s="46"/>
+      <c r="E81" s="46"/>
+      <c r="F81" s="46"/>
+      <c r="G81" s="46"/>
+      <c r="H81" s="46"/>
+      <c r="I81" s="47"/>
     </row>
     <row r="82" spans="3:9">
-      <c r="C82" s="67" t="s">
+      <c r="C82" s="45" t="s">
         <v>497</v>
       </c>
-      <c r="D82" s="68"/>
-      <c r="E82" s="68"/>
-      <c r="F82" s="68"/>
-      <c r="G82" s="68"/>
-      <c r="H82" s="68"/>
-      <c r="I82" s="69"/>
+      <c r="D82" s="46"/>
+      <c r="E82" s="46"/>
+      <c r="F82" s="46"/>
+      <c r="G82" s="46"/>
+      <c r="H82" s="46"/>
+      <c r="I82" s="47"/>
     </row>
     <row r="83" spans="3:9">
-      <c r="C83" s="70"/>
-      <c r="D83" s="68"/>
-      <c r="E83" s="68"/>
-      <c r="F83" s="68"/>
-      <c r="G83" s="68"/>
-      <c r="H83" s="68"/>
-      <c r="I83" s="69"/>
+      <c r="C83" s="48"/>
+      <c r="D83" s="46"/>
+      <c r="E83" s="46"/>
+      <c r="F83" s="46"/>
+      <c r="G83" s="46"/>
+      <c r="H83" s="46"/>
+      <c r="I83" s="47"/>
     </row>
     <row r="84" spans="3:9">
-      <c r="C84" s="67" t="s">
+      <c r="C84" s="45" t="s">
         <v>464</v>
       </c>
-      <c r="D84" s="68"/>
-      <c r="E84" s="68"/>
-      <c r="F84" s="68"/>
-      <c r="G84" s="68"/>
-      <c r="H84" s="68"/>
-      <c r="I84" s="69"/>
+      <c r="D84" s="46"/>
+      <c r="E84" s="46"/>
+      <c r="F84" s="46"/>
+      <c r="G84" s="46"/>
+      <c r="H84" s="46"/>
+      <c r="I84" s="47"/>
     </row>
     <row r="85" spans="3:9">
-      <c r="C85" s="67" t="s">
+      <c r="C85" s="45" t="s">
         <v>465</v>
       </c>
-      <c r="D85" s="68"/>
-      <c r="E85" s="68"/>
-      <c r="F85" s="68"/>
-      <c r="G85" s="68"/>
-      <c r="H85" s="68"/>
-      <c r="I85" s="69"/>
+      <c r="D85" s="46"/>
+      <c r="E85" s="46"/>
+      <c r="F85" s="46"/>
+      <c r="G85" s="46"/>
+      <c r="H85" s="46"/>
+      <c r="I85" s="47"/>
     </row>
     <row r="86" spans="3:9">
-      <c r="C86" s="67" t="s">
+      <c r="C86" s="45" t="s">
         <v>498</v>
       </c>
-      <c r="D86" s="68"/>
-      <c r="E86" s="68"/>
-      <c r="F86" s="68"/>
-      <c r="G86" s="68"/>
-      <c r="H86" s="68"/>
-      <c r="I86" s="69"/>
+      <c r="D86" s="46"/>
+      <c r="E86" s="46"/>
+      <c r="F86" s="46"/>
+      <c r="G86" s="46"/>
+      <c r="H86" s="46"/>
+      <c r="I86" s="47"/>
     </row>
     <row r="87" spans="3:9">
-      <c r="C87" s="71" t="s">
+      <c r="C87" s="49" t="s">
         <v>499</v>
       </c>
-      <c r="D87" s="72"/>
-      <c r="E87" s="72"/>
-      <c r="F87" s="72"/>
-      <c r="G87" s="72"/>
-      <c r="H87" s="72"/>
-      <c r="I87" s="73"/>
-    </row>
-    <row r="122" spans="2:2" ht="15">
+      <c r="D87" s="50"/>
+      <c r="E87" s="50"/>
+      <c r="F87" s="50"/>
+      <c r="G87" s="50"/>
+      <c r="H87" s="50"/>
+      <c r="I87" s="51"/>
+    </row>
+    <row r="122" spans="2:2">
       <c r="B122" s="9"/>
     </row>
     <row r="123" spans="2:2">
@@ -8633,34 +8545,34 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE78E924-1D29-47CA-9F07-3262D21CBE10}">
   <dimension ref="B2:J33"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <sheetData>
-    <row r="2" spans="2:3" ht="23.25">
+    <row r="2" spans="2:3" ht="22.8">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:3" ht="17.25">
+    <row r="3" spans="2:3" ht="17.399999999999999">
       <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:3" ht="15">
+    <row r="4" spans="2:3">
       <c r="C4" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:3" ht="15">
+    <row r="5" spans="2:3">
       <c r="C5" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="2:3" ht="15">
+    <row r="6" spans="2:3">
       <c r="C6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="2:3" ht="17.25">
+    <row r="8" spans="2:3" ht="17.399999999999999">
       <c r="B8" s="2" t="s">
         <v>5</v>
       </c>
@@ -8685,12 +8597,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="2:3" ht="17.25">
+    <row r="14" spans="2:3" ht="17.399999999999999">
       <c r="B14" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="2:3" ht="15">
+    <row r="15" spans="2:3">
       <c r="B15" s="3" t="s">
         <v>11</v>
       </c>
@@ -8715,22 +8627,22 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="2:10" ht="15">
+    <row r="20" spans="2:10">
       <c r="B20" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="2:10" ht="17.25">
+    <row r="22" spans="2:10" ht="17.399999999999999">
       <c r="B22" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="2:10" ht="15">
+    <row r="23" spans="2:10">
       <c r="C23" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="2:10" ht="15">
+    <row r="24" spans="2:10">
       <c r="C24" s="3" t="s">
         <v>19</v>
       </c>
@@ -8745,76 +8657,76 @@
         <v>21</v>
       </c>
     </row>
-    <row r="27" spans="2:10" ht="15">
+    <row r="27" spans="2:10">
       <c r="C27" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="28" spans="2:10" ht="15">
+    <row r="28" spans="2:10">
       <c r="C28" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="29" spans="2:10" ht="23.25">
+    <row r="29" spans="2:10" ht="22.8">
       <c r="B29" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="30" spans="2:10" ht="27.6" customHeight="1">
-      <c r="C30" s="33" t="s">
+      <c r="C30" s="81" t="s">
         <v>25</v>
       </c>
-      <c r="D30" s="33"/>
-      <c r="E30" s="33"/>
-      <c r="F30" s="33"/>
-      <c r="G30" s="33" t="s">
+      <c r="D30" s="81"/>
+      <c r="E30" s="81"/>
+      <c r="F30" s="81"/>
+      <c r="G30" s="81" t="s">
         <v>26</v>
       </c>
-      <c r="H30" s="33"/>
-      <c r="I30" s="33"/>
-      <c r="J30" s="33"/>
+      <c r="H30" s="81"/>
+      <c r="I30" s="81"/>
+      <c r="J30" s="81"/>
     </row>
     <row r="31" spans="2:10">
-      <c r="C31" s="34" t="s">
+      <c r="C31" s="82" t="s">
         <v>27</v>
       </c>
-      <c r="D31" s="34"/>
-      <c r="E31" s="34"/>
-      <c r="F31" s="34"/>
-      <c r="G31" s="34" t="s">
+      <c r="D31" s="82"/>
+      <c r="E31" s="82"/>
+      <c r="F31" s="82"/>
+      <c r="G31" s="82" t="s">
         <v>28</v>
       </c>
-      <c r="H31" s="34"/>
-      <c r="I31" s="34"/>
-      <c r="J31" s="34"/>
+      <c r="H31" s="82"/>
+      <c r="I31" s="82"/>
+      <c r="J31" s="82"/>
     </row>
     <row r="32" spans="2:10">
-      <c r="C32" s="34" t="s">
+      <c r="C32" s="82" t="s">
         <v>29</v>
       </c>
-      <c r="D32" s="34"/>
-      <c r="E32" s="34"/>
-      <c r="F32" s="34"/>
-      <c r="G32" s="34" t="s">
+      <c r="D32" s="82"/>
+      <c r="E32" s="82"/>
+      <c r="F32" s="82"/>
+      <c r="G32" s="82" t="s">
         <v>30</v>
       </c>
-      <c r="H32" s="34"/>
-      <c r="I32" s="34"/>
-      <c r="J32" s="34"/>
+      <c r="H32" s="82"/>
+      <c r="I32" s="82"/>
+      <c r="J32" s="82"/>
     </row>
     <row r="33" spans="3:10">
-      <c r="C33" s="34" t="s">
+      <c r="C33" s="82" t="s">
         <v>31</v>
       </c>
-      <c r="D33" s="34"/>
-      <c r="E33" s="34"/>
-      <c r="F33" s="34"/>
-      <c r="G33" s="34" t="s">
+      <c r="D33" s="82"/>
+      <c r="E33" s="82"/>
+      <c r="F33" s="82"/>
+      <c r="G33" s="82" t="s">
         <v>32</v>
       </c>
-      <c r="H33" s="34"/>
-      <c r="I33" s="34"/>
-      <c r="J33" s="34"/>
+      <c r="H33" s="82"/>
+      <c r="I33" s="82"/>
+      <c r="J33" s="82"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -8835,39 +8747,39 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5FD2A29-D54D-4DFB-98BD-EADAA0E18CB8}">
   <dimension ref="B2:J40"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <sheetData>
-    <row r="2" spans="2:4" ht="23.25">
+    <row r="2" spans="2:4" ht="22.8">
       <c r="B2" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="17.25">
+    <row r="3" spans="2:4" ht="17.399999999999999">
       <c r="B3" s="2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="15">
+    <row r="4" spans="2:4">
       <c r="C4" s="3" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="15">
+    <row r="5" spans="2:4">
       <c r="C5" s="3" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="23.25">
+    <row r="7" spans="2:4" ht="22.8">
       <c r="B7" s="1" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="17.25">
+    <row r="8" spans="2:4" ht="17.399999999999999">
       <c r="C8" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15">
+    <row r="9" spans="2:4">
       <c r="D9" s="3" t="s">
         <v>73</v>
       </c>
@@ -8878,12 +8790,12 @@
         <v>74</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="17.25">
+    <row r="11" spans="2:4" ht="17.399999999999999">
       <c r="B11" s="2" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="12" spans="2:4" ht="15">
+    <row r="12" spans="2:4">
       <c r="B12" s="3"/>
       <c r="C12" s="8" t="s">
         <v>76</v>
@@ -8894,7 +8806,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="15">
+    <row r="14" spans="2:4">
       <c r="C14" s="8" t="s">
         <v>78</v>
       </c>
@@ -8910,22 +8822,22 @@
         <v>80</v>
       </c>
     </row>
-    <row r="18" spans="2:10" ht="23.25">
+    <row r="18" spans="2:10" ht="22.8">
       <c r="B18" s="1" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="19" spans="2:10" ht="17.25">
+    <row r="19" spans="2:10" ht="17.399999999999999">
       <c r="B19" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="20" spans="2:10" ht="15">
+    <row r="20" spans="2:10">
       <c r="C20" s="3" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="21" spans="2:10" ht="15">
+    <row r="21" spans="2:10">
       <c r="C21" s="3" t="s">
         <v>83</v>
       </c>
@@ -8950,82 +8862,82 @@
         <v>87</v>
       </c>
     </row>
-    <row r="27" spans="2:10" ht="23.25">
+    <row r="27" spans="2:10" ht="22.8">
       <c r="B27" s="1" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="29" spans="2:10" ht="30" customHeight="1">
-      <c r="C29" s="33" t="s">
+      <c r="C29" s="81" t="s">
         <v>89</v>
       </c>
-      <c r="D29" s="33"/>
-      <c r="E29" s="33"/>
-      <c r="F29" s="33" t="s">
+      <c r="D29" s="81"/>
+      <c r="E29" s="81"/>
+      <c r="F29" s="81" t="s">
         <v>90</v>
       </c>
-      <c r="G29" s="33"/>
-      <c r="H29" s="33"/>
-      <c r="I29" s="33"/>
-      <c r="J29" s="33"/>
+      <c r="G29" s="81"/>
+      <c r="H29" s="81"/>
+      <c r="I29" s="81"/>
+      <c r="J29" s="81"/>
     </row>
     <row r="30" spans="2:10">
-      <c r="C30" s="35" t="s">
+      <c r="C30" s="83" t="s">
         <v>91</v>
       </c>
-      <c r="D30" s="35"/>
-      <c r="E30" s="35"/>
-      <c r="F30" s="34" t="s">
+      <c r="D30" s="83"/>
+      <c r="E30" s="83"/>
+      <c r="F30" s="82" t="s">
         <v>92</v>
       </c>
-      <c r="G30" s="34"/>
-      <c r="H30" s="34"/>
-      <c r="I30" s="34"/>
-      <c r="J30" s="34"/>
+      <c r="G30" s="82"/>
+      <c r="H30" s="82"/>
+      <c r="I30" s="82"/>
+      <c r="J30" s="82"/>
     </row>
     <row r="31" spans="2:10" ht="36.75" customHeight="1">
-      <c r="C31" s="35" t="s">
+      <c r="C31" s="83" t="s">
         <v>93</v>
       </c>
-      <c r="D31" s="35"/>
-      <c r="E31" s="35"/>
-      <c r="F31" s="34" t="s">
+      <c r="D31" s="83"/>
+      <c r="E31" s="83"/>
+      <c r="F31" s="82" t="s">
         <v>94</v>
       </c>
-      <c r="G31" s="34"/>
-      <c r="H31" s="34"/>
-      <c r="I31" s="34"/>
-      <c r="J31" s="34"/>
+      <c r="G31" s="82"/>
+      <c r="H31" s="82"/>
+      <c r="I31" s="82"/>
+      <c r="J31" s="82"/>
     </row>
     <row r="32" spans="2:10">
-      <c r="C32" s="34" t="s">
+      <c r="C32" s="82" t="s">
         <v>95</v>
       </c>
-      <c r="D32" s="34"/>
-      <c r="E32" s="34"/>
-      <c r="F32" s="35" t="s">
+      <c r="D32" s="82"/>
+      <c r="E32" s="82"/>
+      <c r="F32" s="83" t="s">
         <v>96</v>
       </c>
-      <c r="G32" s="35"/>
-      <c r="H32" s="35"/>
-      <c r="I32" s="35"/>
-      <c r="J32" s="35"/>
+      <c r="G32" s="83"/>
+      <c r="H32" s="83"/>
+      <c r="I32" s="83"/>
+      <c r="J32" s="83"/>
     </row>
     <row r="33" spans="2:10" ht="31.5" customHeight="1">
-      <c r="C33" s="34" t="s">
+      <c r="C33" s="82" t="s">
         <v>97</v>
       </c>
-      <c r="D33" s="34"/>
-      <c r="E33" s="34"/>
-      <c r="F33" s="34" t="s">
+      <c r="D33" s="82"/>
+      <c r="E33" s="82"/>
+      <c r="F33" s="82" t="s">
         <v>98</v>
       </c>
-      <c r="G33" s="34"/>
-      <c r="H33" s="34"/>
-      <c r="I33" s="34"/>
-      <c r="J33" s="34"/>
-    </row>
-    <row r="36" spans="2:10" ht="23.25">
+      <c r="G33" s="82"/>
+      <c r="H33" s="82"/>
+      <c r="I33" s="82"/>
+      <c r="J33" s="82"/>
+    </row>
+    <row r="36" spans="2:10" ht="22.8">
       <c r="B36" s="1"/>
     </row>
     <row r="37" spans="2:10">
@@ -9037,7 +8949,7 @@
     <row r="39" spans="2:10">
       <c r="B39" s="3"/>
     </row>
-    <row r="40" spans="2:10" ht="15">
+    <row r="40" spans="2:10">
       <c r="B40" s="8"/>
     </row>
   </sheetData>
@@ -9060,39 +8972,39 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0DA5883-D5C3-4E46-AF67-539FB53F8190}">
   <dimension ref="B2:D48"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <sheetData>
-    <row r="2" spans="2:4" ht="23.25">
+    <row r="2" spans="2:4" ht="22.8">
       <c r="B2" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="17.25">
+    <row r="3" spans="2:4" ht="17.399999999999999">
       <c r="B3" s="2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="15">
+    <row r="4" spans="2:4">
       <c r="C4" s="8" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="15">
+    <row r="5" spans="2:4">
       <c r="C5" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="17.25">
+    <row r="7" spans="2:4" ht="17.399999999999999">
       <c r="B7" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="15">
+    <row r="8" spans="2:4">
       <c r="C8" s="8" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15">
+    <row r="9" spans="2:4">
       <c r="C9" s="8" t="s">
         <v>39</v>
       </c>
@@ -9102,7 +9014,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="2:4" ht="17.25">
+    <row r="12" spans="2:4" ht="17.399999999999999">
       <c r="B12" s="2" t="s">
         <v>41</v>
       </c>
@@ -9127,7 +9039,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="2:3" ht="17.25">
+    <row r="18" spans="2:3" ht="17.399999999999999">
       <c r="B18" s="2" t="s">
         <v>46</v>
       </c>
@@ -9137,12 +9049,12 @@
         <v>47</v>
       </c>
     </row>
-    <row r="20" spans="2:3" ht="15">
+    <row r="20" spans="2:3">
       <c r="C20" s="8" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="21" spans="2:3" ht="15">
+    <row r="21" spans="2:3">
       <c r="C21" s="3" t="s">
         <v>49</v>
       </c>
@@ -9162,7 +9074,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="25" spans="2:3" ht="17.25">
+    <row r="25" spans="2:3" ht="17.399999999999999">
       <c r="B25" s="2" t="s">
         <v>53</v>
       </c>
@@ -9177,12 +9089,12 @@
         <v>55</v>
       </c>
     </row>
-    <row r="28" spans="2:3" ht="15">
+    <row r="28" spans="2:3">
       <c r="C28" s="3" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="29" spans="2:3" ht="17.25">
+    <row r="29" spans="2:3" ht="17.399999999999999">
       <c r="B29" s="2" t="s">
         <v>57</v>
       </c>
@@ -9212,7 +9124,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="36" spans="2:4" ht="17.25">
+    <row r="36" spans="2:4" ht="17.399999999999999">
       <c r="B36" s="2" t="s">
         <v>63</v>
       </c>
@@ -9232,10 +9144,10 @@
         <v>66</v>
       </c>
     </row>
-    <row r="41" spans="2:4" ht="23.25">
+    <row r="41" spans="2:4" ht="22.8">
       <c r="B41" s="1"/>
     </row>
-    <row r="43" spans="2:4" ht="15">
+    <row r="43" spans="2:4">
       <c r="B43" s="6"/>
       <c r="C43" s="6"/>
       <c r="D43" s="6"/>
@@ -9274,14 +9186,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13D0CC85-3BA6-4A48-8978-56CB9BF6EAF6}">
   <dimension ref="B2:J31"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <sheetData>
-    <row r="2" spans="2:3" ht="23.25">
+    <row r="2" spans="2:3" ht="22.8">
       <c r="B2" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="3" spans="2:3" ht="17.25">
+    <row r="3" spans="2:3" ht="17.399999999999999">
       <c r="B3" s="2" t="s">
         <v>100</v>
       </c>
@@ -9291,17 +9203,17 @@
         <v>101</v>
       </c>
     </row>
-    <row r="5" spans="2:3" ht="15">
+    <row r="5" spans="2:3">
       <c r="B5" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="6" spans="2:3" ht="15">
+    <row r="6" spans="2:3">
       <c r="C6" s="9" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="8" spans="2:3" ht="23.25">
+    <row r="8" spans="2:3" ht="22.8">
       <c r="B8" s="1" t="s">
         <v>104</v>
       </c>
@@ -9311,17 +9223,17 @@
         <v>105</v>
       </c>
     </row>
-    <row r="10" spans="2:3" ht="15">
+    <row r="10" spans="2:3">
       <c r="B10" s="12" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="11" spans="2:3" ht="15">
+    <row r="11" spans="2:3">
       <c r="B11" s="3" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="12" spans="2:3" ht="15">
+    <row r="12" spans="2:3">
       <c r="B12" s="3" t="s">
         <v>108</v>
       </c>
@@ -9351,12 +9263,12 @@
         <v>113</v>
       </c>
     </row>
-    <row r="19" spans="2:10" ht="23.25">
+    <row r="19" spans="2:10" ht="22.8">
       <c r="B19" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="20" spans="2:10" ht="15">
+    <row r="20" spans="2:10">
       <c r="B20" s="8" t="s">
         <v>115</v>
       </c>
@@ -9366,7 +9278,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="22" spans="2:10" ht="15">
+    <row r="22" spans="2:10">
       <c r="B22" s="8" t="s">
         <v>117</v>
       </c>
@@ -9381,80 +9293,80 @@
         <v>119</v>
       </c>
     </row>
-    <row r="25" spans="2:10" ht="23.25">
+    <row r="25" spans="2:10" ht="22.8">
       <c r="B25" s="1" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="27" spans="2:10" ht="15">
-      <c r="C27" s="33" t="s">
+    <row r="27" spans="2:10">
+      <c r="C27" s="81" t="s">
         <v>89</v>
       </c>
-      <c r="D27" s="33"/>
-      <c r="E27" s="33" t="s">
+      <c r="D27" s="81"/>
+      <c r="E27" s="81" t="s">
         <v>90</v>
       </c>
-      <c r="F27" s="33"/>
-      <c r="G27" s="33"/>
-      <c r="H27" s="33"/>
-      <c r="I27" s="33"/>
-      <c r="J27" s="33"/>
-    </row>
-    <row r="28" spans="2:10" ht="15">
-      <c r="C28" s="36" t="s">
+      <c r="F27" s="81"/>
+      <c r="G27" s="81"/>
+      <c r="H27" s="81"/>
+      <c r="I27" s="81"/>
+      <c r="J27" s="81"/>
+    </row>
+    <row r="28" spans="2:10">
+      <c r="C28" s="84" t="s">
         <v>121</v>
       </c>
-      <c r="D28" s="36"/>
-      <c r="E28" s="34" t="s">
+      <c r="D28" s="84"/>
+      <c r="E28" s="82" t="s">
         <v>122</v>
       </c>
-      <c r="F28" s="34"/>
-      <c r="G28" s="34"/>
-      <c r="H28" s="34"/>
-      <c r="I28" s="34"/>
-      <c r="J28" s="34"/>
-    </row>
-    <row r="29" spans="2:10" ht="15">
-      <c r="C29" s="36" t="s">
+      <c r="F28" s="82"/>
+      <c r="G28" s="82"/>
+      <c r="H28" s="82"/>
+      <c r="I28" s="82"/>
+      <c r="J28" s="82"/>
+    </row>
+    <row r="29" spans="2:10">
+      <c r="C29" s="84" t="s">
         <v>123</v>
       </c>
-      <c r="D29" s="36"/>
-      <c r="E29" s="34" t="s">
+      <c r="D29" s="84"/>
+      <c r="E29" s="82" t="s">
         <v>124</v>
       </c>
-      <c r="F29" s="34"/>
-      <c r="G29" s="34"/>
-      <c r="H29" s="34"/>
-      <c r="I29" s="34"/>
-      <c r="J29" s="34"/>
-    </row>
-    <row r="30" spans="2:10" ht="15">
-      <c r="C30" s="36" t="s">
+      <c r="F29" s="82"/>
+      <c r="G29" s="82"/>
+      <c r="H29" s="82"/>
+      <c r="I29" s="82"/>
+      <c r="J29" s="82"/>
+    </row>
+    <row r="30" spans="2:10">
+      <c r="C30" s="84" t="s">
         <v>125</v>
       </c>
-      <c r="D30" s="36"/>
-      <c r="E30" s="34" t="s">
+      <c r="D30" s="84"/>
+      <c r="E30" s="82" t="s">
         <v>126</v>
       </c>
-      <c r="F30" s="34"/>
-      <c r="G30" s="34"/>
-      <c r="H30" s="34"/>
-      <c r="I30" s="34"/>
-      <c r="J30" s="34"/>
+      <c r="F30" s="82"/>
+      <c r="G30" s="82"/>
+      <c r="H30" s="82"/>
+      <c r="I30" s="82"/>
+      <c r="J30" s="82"/>
     </row>
     <row r="31" spans="2:10" ht="32.25" customHeight="1">
-      <c r="C31" s="36" t="s">
+      <c r="C31" s="84" t="s">
         <v>127</v>
       </c>
-      <c r="D31" s="36"/>
-      <c r="E31" s="34" t="s">
+      <c r="D31" s="84"/>
+      <c r="E31" s="82" t="s">
         <v>128</v>
       </c>
-      <c r="F31" s="34"/>
-      <c r="G31" s="34"/>
-      <c r="H31" s="34"/>
-      <c r="I31" s="34"/>
-      <c r="J31" s="34"/>
+      <c r="F31" s="82"/>
+      <c r="G31" s="82"/>
+      <c r="H31" s="82"/>
+      <c r="I31" s="82"/>
+      <c r="J31" s="82"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -9476,15 +9388,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C212CEFC-7EA5-425F-BDF2-54E0CCD3335D}">
   <dimension ref="B3:Z79"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="15" max="15" width="1.625" customWidth="1"/>
+    <col min="15" max="15" width="1.59765625" customWidth="1"/>
     <col min="17" max="17" width="5" customWidth="1"/>
-    <col min="21" max="21" width="6.875" customWidth="1"/>
+    <col min="21" max="21" width="6.8984375" customWidth="1"/>
     <col min="22" max="22" width="9" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:4" ht="23.25">
+    <row r="3" spans="2:4" ht="22.8">
       <c r="B3" s="1" t="s">
         <v>129</v>
       </c>
@@ -9494,7 +9406,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15">
+    <row r="6" spans="2:4">
       <c r="C6" s="14" t="s">
         <v>131</v>
       </c>
@@ -9509,7 +9421,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="15.75">
+    <row r="10" spans="2:4" ht="15.6">
       <c r="C10" s="15" t="s">
         <v>134</v>
       </c>
@@ -9524,7 +9436,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="15.75">
+    <row r="13" spans="2:4" ht="15.6">
       <c r="C13" s="15" t="s">
         <v>137</v>
       </c>
@@ -9539,7 +9451,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="16" spans="2:4" ht="15.75">
+    <row r="16" spans="2:4" ht="15.6">
       <c r="C16" s="15" t="s">
         <v>140</v>
       </c>
@@ -9559,12 +9471,12 @@
         <v>143</v>
       </c>
     </row>
-    <row r="20" spans="2:26" ht="15">
+    <row r="20" spans="2:26">
       <c r="D20" s="3" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="21" spans="2:26" ht="17.25">
+    <row r="21" spans="2:26" ht="17.399999999999999">
       <c r="B21" s="2" t="s">
         <v>145</v>
       </c>
@@ -9574,12 +9486,12 @@
         <v>142</v>
       </c>
     </row>
-    <row r="23" spans="2:26" ht="15">
+    <row r="23" spans="2:26">
       <c r="C23" s="16" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="24" spans="2:26" ht="15">
+    <row r="24" spans="2:26">
       <c r="C24" s="16" t="s">
         <v>147</v>
       </c>
@@ -9590,221 +9502,221 @@
         <v>148</v>
       </c>
     </row>
-    <row r="26" spans="2:26" ht="15">
+    <row r="26" spans="2:26">
       <c r="D26" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="K26" s="38" t="s">
+      <c r="K26" s="86" t="s">
         <v>151</v>
       </c>
-      <c r="L26" s="38"/>
-      <c r="M26" s="38" t="s">
+      <c r="L26" s="86"/>
+      <c r="M26" s="86" t="s">
         <v>152</v>
       </c>
-      <c r="N26" s="38"/>
-      <c r="O26" s="38"/>
-      <c r="P26" s="38" t="s">
+      <c r="N26" s="86"/>
+      <c r="O26" s="86"/>
+      <c r="P26" s="86" t="s">
         <v>153</v>
       </c>
-      <c r="Q26" s="38"/>
-      <c r="R26" s="38" t="s">
+      <c r="Q26" s="86"/>
+      <c r="R26" s="86" t="s">
         <v>154</v>
       </c>
-      <c r="S26" s="38"/>
-      <c r="T26" s="38"/>
-      <c r="U26" s="38"/>
-      <c r="V26" s="38"/>
-      <c r="W26" s="38" t="s">
+      <c r="S26" s="86"/>
+      <c r="T26" s="86"/>
+      <c r="U26" s="86"/>
+      <c r="V26" s="86"/>
+      <c r="W26" s="86" t="s">
         <v>155</v>
       </c>
-      <c r="X26" s="38"/>
-      <c r="Y26" s="38"/>
-      <c r="Z26" s="38"/>
-    </row>
-    <row r="27" spans="2:26" ht="15">
+      <c r="X26" s="86"/>
+      <c r="Y26" s="86"/>
+      <c r="Z26" s="86"/>
+    </row>
+    <row r="27" spans="2:26">
       <c r="C27" s="5"/>
-      <c r="K27" s="39" t="s">
+      <c r="K27" s="87" t="s">
         <v>156</v>
       </c>
-      <c r="L27" s="39"/>
-      <c r="M27" s="42" t="s">
+      <c r="L27" s="87"/>
+      <c r="M27" s="90" t="s">
         <v>157</v>
       </c>
-      <c r="N27" s="42"/>
-      <c r="O27" s="42"/>
-      <c r="P27" s="40" t="s">
+      <c r="N27" s="90"/>
+      <c r="O27" s="90"/>
+      <c r="P27" s="88" t="s">
         <v>158</v>
       </c>
-      <c r="Q27" s="40"/>
-      <c r="R27" s="40" t="s">
+      <c r="Q27" s="88"/>
+      <c r="R27" s="88" t="s">
         <v>159</v>
       </c>
-      <c r="S27" s="40"/>
-      <c r="T27" s="40"/>
-      <c r="U27" s="40"/>
-      <c r="V27" s="40"/>
-      <c r="W27" s="40" t="s">
+      <c r="S27" s="88"/>
+      <c r="T27" s="88"/>
+      <c r="U27" s="88"/>
+      <c r="V27" s="88"/>
+      <c r="W27" s="88" t="s">
         <v>160</v>
       </c>
-      <c r="X27" s="40"/>
-      <c r="Y27" s="40"/>
-      <c r="Z27" s="40"/>
-    </row>
-    <row r="28" spans="2:26" ht="17.25">
+      <c r="X27" s="88"/>
+      <c r="Y27" s="88"/>
+      <c r="Z27" s="88"/>
+    </row>
+    <row r="28" spans="2:26" ht="17.399999999999999">
       <c r="B28" s="2"/>
-      <c r="K28" s="39" t="s">
+      <c r="K28" s="87" t="s">
         <v>161</v>
       </c>
-      <c r="L28" s="39"/>
-      <c r="M28" s="42" t="s">
+      <c r="L28" s="87"/>
+      <c r="M28" s="90" t="s">
         <v>162</v>
       </c>
-      <c r="N28" s="42"/>
-      <c r="O28" s="42"/>
-      <c r="P28" s="40" t="s">
+      <c r="N28" s="90"/>
+      <c r="O28" s="90"/>
+      <c r="P28" s="88" t="s">
         <v>163</v>
       </c>
-      <c r="Q28" s="40"/>
-      <c r="R28" s="40" t="s">
+      <c r="Q28" s="88"/>
+      <c r="R28" s="88" t="s">
         <v>164</v>
       </c>
-      <c r="S28" s="40"/>
-      <c r="T28" s="40"/>
-      <c r="U28" s="40"/>
-      <c r="V28" s="40"/>
-      <c r="W28" s="40" t="s">
+      <c r="S28" s="88"/>
+      <c r="T28" s="88"/>
+      <c r="U28" s="88"/>
+      <c r="V28" s="88"/>
+      <c r="W28" s="88" t="s">
         <v>165</v>
       </c>
-      <c r="X28" s="40"/>
-      <c r="Y28" s="40"/>
-      <c r="Z28" s="40"/>
-    </row>
-    <row r="29" spans="2:26" ht="15">
+      <c r="X28" s="88"/>
+      <c r="Y28" s="88"/>
+      <c r="Z28" s="88"/>
+    </row>
+    <row r="29" spans="2:26">
       <c r="C29" s="3"/>
-      <c r="K29" s="39" t="s">
+      <c r="K29" s="87" t="s">
         <v>166</v>
       </c>
-      <c r="L29" s="39"/>
-      <c r="M29" s="42" t="s">
+      <c r="L29" s="87"/>
+      <c r="M29" s="90" t="s">
         <v>167</v>
       </c>
-      <c r="N29" s="42"/>
-      <c r="O29" s="42"/>
-      <c r="P29" s="40" t="s">
+      <c r="N29" s="90"/>
+      <c r="O29" s="90"/>
+      <c r="P29" s="88" t="s">
         <v>168</v>
       </c>
-      <c r="Q29" s="40"/>
-      <c r="R29" s="42" t="s">
+      <c r="Q29" s="88"/>
+      <c r="R29" s="90" t="s">
         <v>169</v>
       </c>
-      <c r="S29" s="42"/>
-      <c r="T29" s="42"/>
-      <c r="U29" s="42"/>
-      <c r="V29" s="42"/>
-      <c r="W29" s="40" t="s">
+      <c r="S29" s="90"/>
+      <c r="T29" s="90"/>
+      <c r="U29" s="90"/>
+      <c r="V29" s="90"/>
+      <c r="W29" s="88" t="s">
         <v>170</v>
       </c>
-      <c r="X29" s="40"/>
-      <c r="Y29" s="40"/>
-      <c r="Z29" s="40"/>
-    </row>
-    <row r="30" spans="2:26" ht="15">
+      <c r="X29" s="88"/>
+      <c r="Y29" s="88"/>
+      <c r="Z29" s="88"/>
+    </row>
+    <row r="30" spans="2:26">
       <c r="B30" s="4"/>
-      <c r="K30" s="39" t="s">
+      <c r="K30" s="87" t="s">
         <v>171</v>
       </c>
-      <c r="L30" s="39"/>
-      <c r="M30" s="42" t="s">
+      <c r="L30" s="87"/>
+      <c r="M30" s="90" t="s">
         <v>172</v>
       </c>
-      <c r="N30" s="42"/>
-      <c r="O30" s="42"/>
-      <c r="P30" s="40" t="s">
+      <c r="N30" s="90"/>
+      <c r="O30" s="90"/>
+      <c r="P30" s="88" t="s">
         <v>173</v>
       </c>
-      <c r="Q30" s="40"/>
-      <c r="R30" s="40" t="s">
+      <c r="Q30" s="88"/>
+      <c r="R30" s="88" t="s">
         <v>174</v>
       </c>
-      <c r="S30" s="40"/>
-      <c r="T30" s="40"/>
-      <c r="U30" s="40"/>
-      <c r="V30" s="40"/>
-      <c r="W30" s="40" t="s">
+      <c r="S30" s="88"/>
+      <c r="T30" s="88"/>
+      <c r="U30" s="88"/>
+      <c r="V30" s="88"/>
+      <c r="W30" s="88" t="s">
         <v>175</v>
       </c>
-      <c r="X30" s="40"/>
-      <c r="Y30" s="40"/>
-      <c r="Z30" s="40"/>
-    </row>
-    <row r="31" spans="2:26" ht="15">
+      <c r="X30" s="88"/>
+      <c r="Y30" s="88"/>
+      <c r="Z30" s="88"/>
+    </row>
+    <row r="31" spans="2:26">
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
-      <c r="K31" s="39" t="s">
+      <c r="K31" s="87" t="s">
         <v>176</v>
       </c>
-      <c r="L31" s="39"/>
-      <c r="M31" s="42" t="s">
+      <c r="L31" s="87"/>
+      <c r="M31" s="90" t="s">
         <v>177</v>
       </c>
-      <c r="N31" s="42"/>
-      <c r="O31" s="42"/>
-      <c r="P31" s="40" t="s">
+      <c r="N31" s="90"/>
+      <c r="O31" s="90"/>
+      <c r="P31" s="88" t="s">
         <v>178</v>
       </c>
-      <c r="Q31" s="40"/>
-      <c r="R31" s="40" t="s">
+      <c r="Q31" s="88"/>
+      <c r="R31" s="88" t="s">
         <v>179</v>
       </c>
-      <c r="S31" s="40"/>
-      <c r="T31" s="40"/>
-      <c r="U31" s="40"/>
-      <c r="V31" s="40"/>
-      <c r="W31" s="40" t="s">
+      <c r="S31" s="88"/>
+      <c r="T31" s="88"/>
+      <c r="U31" s="88"/>
+      <c r="V31" s="88"/>
+      <c r="W31" s="88" t="s">
         <v>150</v>
       </c>
-      <c r="X31" s="40"/>
-      <c r="Y31" s="40"/>
-      <c r="Z31" s="40"/>
-    </row>
-    <row r="32" spans="2:26" ht="15">
+      <c r="X31" s="88"/>
+      <c r="Y31" s="88"/>
+      <c r="Z31" s="88"/>
+    </row>
+    <row r="32" spans="2:26">
       <c r="B32" s="10"/>
       <c r="C32" s="3"/>
-      <c r="K32" s="37" t="s">
+      <c r="K32" s="85" t="s">
         <v>180</v>
       </c>
-      <c r="L32" s="37"/>
-      <c r="M32" s="44" t="s">
+      <c r="L32" s="85"/>
+      <c r="M32" s="92" t="s">
         <v>181</v>
       </c>
-      <c r="N32" s="44"/>
-      <c r="O32" s="44"/>
-      <c r="P32" s="41" t="s">
+      <c r="N32" s="92"/>
+      <c r="O32" s="92"/>
+      <c r="P32" s="89" t="s">
         <v>182</v>
       </c>
-      <c r="Q32" s="41"/>
-      <c r="R32" s="44" t="s">
+      <c r="Q32" s="89"/>
+      <c r="R32" s="92" t="s">
         <v>183</v>
       </c>
-      <c r="S32" s="44"/>
-      <c r="T32" s="44"/>
-      <c r="U32" s="44"/>
-      <c r="V32" s="44"/>
-      <c r="W32" s="41" t="s">
+      <c r="S32" s="92"/>
+      <c r="T32" s="92"/>
+      <c r="U32" s="92"/>
+      <c r="V32" s="92"/>
+      <c r="W32" s="89" t="s">
         <v>184</v>
       </c>
-      <c r="X32" s="41"/>
-      <c r="Y32" s="41"/>
-      <c r="Z32" s="41"/>
+      <c r="X32" s="89"/>
+      <c r="Y32" s="89"/>
+      <c r="Z32" s="89"/>
     </row>
     <row r="33" spans="2:26">
       <c r="B33" s="3"/>
       <c r="C33" s="5"/>
       <c r="K33" s="17"/>
       <c r="L33" s="17"/>
-      <c r="M33" s="45"/>
-      <c r="N33" s="45"/>
-      <c r="O33" s="45"/>
+      <c r="M33" s="93"/>
+      <c r="N33" s="93"/>
+      <c r="O33" s="93"/>
       <c r="P33" s="17"/>
       <c r="Q33" s="17"/>
       <c r="R33" s="17"/>
@@ -9817,332 +9729,332 @@
       <c r="Y33" s="17"/>
       <c r="Z33" s="17"/>
     </row>
-    <row r="34" spans="2:26" ht="15">
+    <row r="34" spans="2:26">
       <c r="B34" s="3"/>
-      <c r="D34" s="43" t="s">
+      <c r="D34" s="91" t="s">
         <v>185</v>
       </c>
-      <c r="E34" s="43"/>
-      <c r="F34" s="43" t="s">
+      <c r="E34" s="91"/>
+      <c r="F34" s="91" t="s">
         <v>151</v>
       </c>
-      <c r="G34" s="43"/>
-      <c r="H34" s="43" t="s">
+      <c r="G34" s="91"/>
+      <c r="H34" s="91" t="s">
         <v>186</v>
       </c>
-      <c r="I34" s="43"/>
-      <c r="J34" s="43"/>
-      <c r="K34" s="43"/>
-      <c r="L34" s="43"/>
-      <c r="M34" s="43"/>
-      <c r="N34" s="43"/>
-      <c r="O34" s="43"/>
-      <c r="P34" s="43"/>
+      <c r="I34" s="91"/>
+      <c r="J34" s="91"/>
+      <c r="K34" s="91"/>
+      <c r="L34" s="91"/>
+      <c r="M34" s="91"/>
+      <c r="N34" s="91"/>
+      <c r="O34" s="91"/>
+      <c r="P34" s="91"/>
     </row>
     <row r="35" spans="2:26">
-      <c r="D35" s="47" t="s">
+      <c r="D35" s="95" t="s">
         <v>187</v>
       </c>
-      <c r="E35" s="47"/>
-      <c r="F35" s="46" t="s">
+      <c r="E35" s="95"/>
+      <c r="F35" s="94" t="s">
         <v>161</v>
       </c>
-      <c r="G35" s="46"/>
-      <c r="H35" s="46" t="s">
+      <c r="G35" s="94"/>
+      <c r="H35" s="94" t="s">
         <v>188</v>
       </c>
-      <c r="I35" s="46"/>
-      <c r="J35" s="46"/>
-      <c r="K35" s="46"/>
-      <c r="L35" s="46"/>
-      <c r="M35" s="46"/>
-      <c r="N35" s="46"/>
-      <c r="O35" s="46"/>
-      <c r="P35" s="46"/>
+      <c r="I35" s="94"/>
+      <c r="J35" s="94"/>
+      <c r="K35" s="94"/>
+      <c r="L35" s="94"/>
+      <c r="M35" s="94"/>
+      <c r="N35" s="94"/>
+      <c r="O35" s="94"/>
+      <c r="P35" s="94"/>
     </row>
     <row r="36" spans="2:26">
-      <c r="D36" s="47" t="s">
+      <c r="D36" s="95" t="s">
         <v>189</v>
       </c>
-      <c r="E36" s="47"/>
-      <c r="F36" s="46" t="s">
+      <c r="E36" s="95"/>
+      <c r="F36" s="94" t="s">
         <v>156</v>
       </c>
-      <c r="G36" s="46"/>
-      <c r="H36" s="47" t="s">
+      <c r="G36" s="94"/>
+      <c r="H36" s="95" t="s">
         <v>190</v>
       </c>
-      <c r="I36" s="47"/>
-      <c r="J36" s="47"/>
-      <c r="K36" s="47"/>
-      <c r="L36" s="47"/>
-      <c r="M36" s="47"/>
-      <c r="N36" s="47"/>
-      <c r="O36" s="47"/>
-      <c r="P36" s="47"/>
+      <c r="I36" s="95"/>
+      <c r="J36" s="95"/>
+      <c r="K36" s="95"/>
+      <c r="L36" s="95"/>
+      <c r="M36" s="95"/>
+      <c r="N36" s="95"/>
+      <c r="O36" s="95"/>
+      <c r="P36" s="95"/>
     </row>
     <row r="37" spans="2:26">
-      <c r="D37" s="47" t="s">
+      <c r="D37" s="95" t="s">
         <v>191</v>
       </c>
-      <c r="E37" s="47"/>
-      <c r="F37" s="46" t="s">
+      <c r="E37" s="95"/>
+      <c r="F37" s="94" t="s">
         <v>192</v>
       </c>
-      <c r="G37" s="46"/>
-      <c r="H37" s="46" t="s">
+      <c r="G37" s="94"/>
+      <c r="H37" s="94" t="s">
         <v>193</v>
       </c>
-      <c r="I37" s="46"/>
-      <c r="J37" s="46"/>
-      <c r="K37" s="46"/>
-      <c r="L37" s="46"/>
-      <c r="M37" s="46"/>
-      <c r="N37" s="46"/>
-      <c r="O37" s="46"/>
-      <c r="P37" s="46"/>
-    </row>
-    <row r="38" spans="2:26" ht="17.25">
+      <c r="I37" s="94"/>
+      <c r="J37" s="94"/>
+      <c r="K37" s="94"/>
+      <c r="L37" s="94"/>
+      <c r="M37" s="94"/>
+      <c r="N37" s="94"/>
+      <c r="O37" s="94"/>
+      <c r="P37" s="94"/>
+    </row>
+    <row r="38" spans="2:26" ht="17.399999999999999">
       <c r="B38" s="2"/>
-      <c r="D38" s="47" t="s">
+      <c r="D38" s="95" t="s">
         <v>194</v>
       </c>
-      <c r="E38" s="47"/>
-      <c r="F38" s="46" t="s">
+      <c r="E38" s="95"/>
+      <c r="F38" s="94" t="s">
         <v>192</v>
       </c>
-      <c r="G38" s="46"/>
-      <c r="H38" s="46" t="s">
+      <c r="G38" s="94"/>
+      <c r="H38" s="94" t="s">
         <v>195</v>
       </c>
-      <c r="I38" s="46"/>
-      <c r="J38" s="46"/>
-      <c r="K38" s="46"/>
-      <c r="L38" s="46"/>
-      <c r="M38" s="46"/>
-      <c r="N38" s="46"/>
-      <c r="O38" s="46"/>
-      <c r="P38" s="46"/>
+      <c r="I38" s="94"/>
+      <c r="J38" s="94"/>
+      <c r="K38" s="94"/>
+      <c r="L38" s="94"/>
+      <c r="M38" s="94"/>
+      <c r="N38" s="94"/>
+      <c r="O38" s="94"/>
+      <c r="P38" s="94"/>
     </row>
     <row r="39" spans="2:26">
-      <c r="D39" s="47" t="s">
+      <c r="D39" s="95" t="s">
         <v>196</v>
       </c>
-      <c r="E39" s="47"/>
-      <c r="F39" s="46" t="s">
+      <c r="E39" s="95"/>
+      <c r="F39" s="94" t="s">
         <v>176</v>
       </c>
-      <c r="G39" s="46"/>
-      <c r="H39" s="46" t="s">
+      <c r="G39" s="94"/>
+      <c r="H39" s="94" t="s">
         <v>197</v>
       </c>
-      <c r="I39" s="46"/>
-      <c r="J39" s="46"/>
-      <c r="K39" s="46"/>
-      <c r="L39" s="46"/>
-      <c r="M39" s="46"/>
-      <c r="N39" s="46"/>
-      <c r="O39" s="46"/>
-      <c r="P39" s="46"/>
+      <c r="I39" s="94"/>
+      <c r="J39" s="94"/>
+      <c r="K39" s="94"/>
+      <c r="L39" s="94"/>
+      <c r="M39" s="94"/>
+      <c r="N39" s="94"/>
+      <c r="O39" s="94"/>
+      <c r="P39" s="94"/>
     </row>
     <row r="40" spans="2:26">
       <c r="B40" s="4"/>
-      <c r="D40" s="47" t="s">
+      <c r="D40" s="95" t="s">
         <v>198</v>
       </c>
-      <c r="E40" s="47"/>
-      <c r="F40" s="46" t="s">
+      <c r="E40" s="95"/>
+      <c r="F40" s="94" t="s">
         <v>199</v>
       </c>
-      <c r="G40" s="46"/>
-      <c r="H40" s="46" t="s">
+      <c r="G40" s="94"/>
+      <c r="H40" s="94" t="s">
         <v>200</v>
       </c>
-      <c r="I40" s="46"/>
-      <c r="J40" s="46"/>
-      <c r="K40" s="46"/>
-      <c r="L40" s="46"/>
-      <c r="M40" s="46"/>
-      <c r="N40" s="46"/>
-      <c r="O40" s="46"/>
-      <c r="P40" s="46"/>
+      <c r="I40" s="94"/>
+      <c r="J40" s="94"/>
+      <c r="K40" s="94"/>
+      <c r="L40" s="94"/>
+      <c r="M40" s="94"/>
+      <c r="N40" s="94"/>
+      <c r="O40" s="94"/>
+      <c r="P40" s="94"/>
     </row>
     <row r="41" spans="2:26">
       <c r="B41" s="3"/>
-      <c r="D41" s="47" t="s">
+      <c r="D41" s="95" t="s">
         <v>201</v>
       </c>
-      <c r="E41" s="47"/>
-      <c r="F41" s="46" t="s">
+      <c r="E41" s="95"/>
+      <c r="F41" s="94" t="s">
         <v>161</v>
       </c>
-      <c r="G41" s="46"/>
-      <c r="H41" s="46" t="s">
+      <c r="G41" s="94"/>
+      <c r="H41" s="94" t="s">
         <v>202</v>
       </c>
-      <c r="I41" s="46"/>
-      <c r="J41" s="46"/>
-      <c r="K41" s="46"/>
-      <c r="L41" s="46"/>
-      <c r="M41" s="46"/>
-      <c r="N41" s="46"/>
-      <c r="O41" s="46"/>
-      <c r="P41" s="46"/>
+      <c r="I41" s="94"/>
+      <c r="J41" s="94"/>
+      <c r="K41" s="94"/>
+      <c r="L41" s="94"/>
+      <c r="M41" s="94"/>
+      <c r="N41" s="94"/>
+      <c r="O41" s="94"/>
+      <c r="P41" s="94"/>
     </row>
     <row r="42" spans="2:26">
       <c r="B42" s="10"/>
-      <c r="D42" s="47" t="s">
+      <c r="D42" s="95" t="s">
         <v>203</v>
       </c>
-      <c r="E42" s="47"/>
-      <c r="F42" s="46" t="s">
+      <c r="E42" s="95"/>
+      <c r="F42" s="94" t="s">
         <v>204</v>
       </c>
-      <c r="G42" s="46"/>
-      <c r="H42" s="46" t="s">
+      <c r="G42" s="94"/>
+      <c r="H42" s="94" t="s">
         <v>205</v>
       </c>
-      <c r="I42" s="46"/>
-      <c r="J42" s="46"/>
-      <c r="K42" s="46"/>
-      <c r="L42" s="46"/>
-      <c r="M42" s="46"/>
-      <c r="N42" s="46"/>
-      <c r="O42" s="46"/>
-      <c r="P42" s="46"/>
+      <c r="I42" s="94"/>
+      <c r="J42" s="94"/>
+      <c r="K42" s="94"/>
+      <c r="L42" s="94"/>
+      <c r="M42" s="94"/>
+      <c r="N42" s="94"/>
+      <c r="O42" s="94"/>
+      <c r="P42" s="94"/>
     </row>
     <row r="43" spans="2:26">
       <c r="B43" s="3"/>
-      <c r="D43" s="47" t="s">
+      <c r="D43" s="95" t="s">
         <v>206</v>
       </c>
-      <c r="E43" s="47"/>
-      <c r="F43" s="46" t="s">
+      <c r="E43" s="95"/>
+      <c r="F43" s="94" t="s">
         <v>207</v>
       </c>
-      <c r="G43" s="46"/>
-      <c r="H43" s="46" t="s">
+      <c r="G43" s="94"/>
+      <c r="H43" s="94" t="s">
         <v>208</v>
       </c>
-      <c r="I43" s="46"/>
-      <c r="J43" s="46"/>
-      <c r="K43" s="46"/>
-      <c r="L43" s="46"/>
-      <c r="M43" s="46"/>
-      <c r="N43" s="46"/>
-      <c r="O43" s="46"/>
-      <c r="P43" s="46"/>
+      <c r="I43" s="94"/>
+      <c r="J43" s="94"/>
+      <c r="K43" s="94"/>
+      <c r="L43" s="94"/>
+      <c r="M43" s="94"/>
+      <c r="N43" s="94"/>
+      <c r="O43" s="94"/>
+      <c r="P43" s="94"/>
     </row>
     <row r="44" spans="2:26">
       <c r="B44" s="3"/>
-      <c r="D44" s="47" t="s">
+      <c r="D44" s="95" t="s">
         <v>209</v>
       </c>
-      <c r="E44" s="47"/>
-      <c r="F44" s="46" t="s">
+      <c r="E44" s="95"/>
+      <c r="F44" s="94" t="s">
         <v>210</v>
       </c>
-      <c r="G44" s="46"/>
-      <c r="H44" s="46" t="s">
+      <c r="G44" s="94"/>
+      <c r="H44" s="94" t="s">
         <v>211</v>
       </c>
-      <c r="I44" s="46"/>
-      <c r="J44" s="46"/>
-      <c r="K44" s="46"/>
-      <c r="L44" s="46"/>
-      <c r="M44" s="46"/>
-      <c r="N44" s="46"/>
-      <c r="O44" s="46"/>
-      <c r="P44" s="46"/>
+      <c r="I44" s="94"/>
+      <c r="J44" s="94"/>
+      <c r="K44" s="94"/>
+      <c r="L44" s="94"/>
+      <c r="M44" s="94"/>
+      <c r="N44" s="94"/>
+      <c r="O44" s="94"/>
+      <c r="P44" s="94"/>
     </row>
     <row r="45" spans="2:26" ht="33.75" customHeight="1">
       <c r="B45" s="3"/>
-      <c r="D45" s="47" t="s">
+      <c r="D45" s="95" t="s">
         <v>212</v>
       </c>
-      <c r="E45" s="47"/>
-      <c r="F45" s="46" t="s">
+      <c r="E45" s="95"/>
+      <c r="F45" s="94" t="s">
         <v>213</v>
       </c>
-      <c r="G45" s="46"/>
-      <c r="H45" s="46" t="s">
+      <c r="G45" s="94"/>
+      <c r="H45" s="94" t="s">
         <v>214</v>
       </c>
-      <c r="I45" s="46"/>
-      <c r="J45" s="46"/>
-      <c r="K45" s="46"/>
-      <c r="L45" s="46"/>
-      <c r="M45" s="46"/>
-      <c r="N45" s="46"/>
-      <c r="O45" s="46"/>
-      <c r="P45" s="46"/>
+      <c r="I45" s="94"/>
+      <c r="J45" s="94"/>
+      <c r="K45" s="94"/>
+      <c r="L45" s="94"/>
+      <c r="M45" s="94"/>
+      <c r="N45" s="94"/>
+      <c r="O45" s="94"/>
+      <c r="P45" s="94"/>
     </row>
     <row r="46" spans="2:26">
       <c r="B46" s="10"/>
-      <c r="D46" s="47" t="s">
+      <c r="D46" s="95" t="s">
         <v>215</v>
       </c>
-      <c r="E46" s="47"/>
-      <c r="F46" s="46" t="s">
+      <c r="E46" s="95"/>
+      <c r="F46" s="94" t="s">
         <v>192</v>
       </c>
-      <c r="G46" s="46"/>
-      <c r="H46" s="46" t="s">
+      <c r="G46" s="94"/>
+      <c r="H46" s="94" t="s">
         <v>216</v>
       </c>
-      <c r="I46" s="46"/>
-      <c r="J46" s="46"/>
-      <c r="K46" s="46"/>
-      <c r="L46" s="46"/>
-      <c r="M46" s="46"/>
-      <c r="N46" s="46"/>
-      <c r="O46" s="46"/>
-      <c r="P46" s="46"/>
+      <c r="I46" s="94"/>
+      <c r="J46" s="94"/>
+      <c r="K46" s="94"/>
+      <c r="L46" s="94"/>
+      <c r="M46" s="94"/>
+      <c r="N46" s="94"/>
+      <c r="O46" s="94"/>
+      <c r="P46" s="94"/>
     </row>
     <row r="47" spans="2:26">
       <c r="B47" s="10"/>
-      <c r="D47" s="47" t="s">
+      <c r="D47" s="95" t="s">
         <v>217</v>
       </c>
-      <c r="E47" s="47"/>
-      <c r="F47" s="46" t="s">
+      <c r="E47" s="95"/>
+      <c r="F47" s="94" t="s">
         <v>166</v>
       </c>
-      <c r="G47" s="46"/>
-      <c r="H47" s="46" t="s">
+      <c r="G47" s="94"/>
+      <c r="H47" s="94" t="s">
         <v>218</v>
       </c>
-      <c r="I47" s="46"/>
-      <c r="J47" s="46"/>
-      <c r="K47" s="46"/>
-      <c r="L47" s="46"/>
-      <c r="M47" s="46"/>
-      <c r="N47" s="46"/>
-      <c r="O47" s="46"/>
-      <c r="P47" s="46"/>
+      <c r="I47" s="94"/>
+      <c r="J47" s="94"/>
+      <c r="K47" s="94"/>
+      <c r="L47" s="94"/>
+      <c r="M47" s="94"/>
+      <c r="N47" s="94"/>
+      <c r="O47" s="94"/>
+      <c r="P47" s="94"/>
     </row>
     <row r="48" spans="2:26">
-      <c r="D48" s="47" t="s">
+      <c r="D48" s="95" t="s">
         <v>219</v>
       </c>
-      <c r="E48" s="47"/>
-      <c r="F48" s="46" t="s">
+      <c r="E48" s="95"/>
+      <c r="F48" s="94" t="s">
         <v>156</v>
       </c>
-      <c r="G48" s="46"/>
-      <c r="H48" s="46" t="s">
+      <c r="G48" s="94"/>
+      <c r="H48" s="94" t="s">
         <v>220</v>
       </c>
-      <c r="I48" s="46"/>
-      <c r="J48" s="46"/>
-      <c r="K48" s="46"/>
-      <c r="L48" s="46"/>
-      <c r="M48" s="46"/>
-      <c r="N48" s="46"/>
-      <c r="O48" s="46"/>
-      <c r="P48" s="46"/>
-    </row>
-    <row r="51" spans="2:2" ht="17.25">
+      <c r="I48" s="94"/>
+      <c r="J48" s="94"/>
+      <c r="K48" s="94"/>
+      <c r="L48" s="94"/>
+      <c r="M48" s="94"/>
+      <c r="N48" s="94"/>
+      <c r="O48" s="94"/>
+      <c r="P48" s="94"/>
+    </row>
+    <row r="51" spans="2:2" ht="17.399999999999999">
       <c r="B51" s="2"/>
     </row>
     <row r="53" spans="2:2">
@@ -10160,7 +10072,7 @@
     <row r="57" spans="2:2">
       <c r="B57" s="3"/>
     </row>
-    <row r="61" spans="2:2" ht="17.25">
+    <row r="61" spans="2:2" ht="17.399999999999999">
       <c r="B61" s="2"/>
     </row>
     <row r="63" spans="2:2">
@@ -10178,25 +10090,25 @@
     <row r="67" spans="2:2">
       <c r="B67" s="3"/>
     </row>
-    <row r="71" spans="2:2" ht="23.25">
+    <row r="71" spans="2:2" ht="22.8">
       <c r="B71" s="1"/>
     </row>
     <row r="74" spans="2:2">
       <c r="B74" s="3"/>
     </row>
-    <row r="75" spans="2:2" ht="15">
+    <row r="75" spans="2:2">
       <c r="B75" s="8"/>
     </row>
     <row r="76" spans="2:2">
       <c r="B76" s="3"/>
     </row>
-    <row r="77" spans="2:2" ht="15">
+    <row r="77" spans="2:2">
       <c r="B77" s="8"/>
     </row>
     <row r="78" spans="2:2">
       <c r="B78" s="3"/>
     </row>
-    <row r="79" spans="2:2" ht="15">
+    <row r="79" spans="2:2">
       <c r="B79" s="8"/>
     </row>
   </sheetData>
@@ -10291,76 +10203,76 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FA746B1-DD43-4413-8C18-9030CB13A504}">
   <dimension ref="B1:W29"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <sheetData>
-    <row r="1" spans="2:23" ht="23.25">
+    <row r="1" spans="2:23" ht="22.8">
       <c r="B1" s="1" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="2" spans="2:23" ht="30">
+    <row r="2" spans="2:23" ht="27.6">
       <c r="B2" s="2" t="s">
         <v>222</v>
       </c>
       <c r="Q2" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="R2" s="48" t="s">
+      <c r="R2" s="96" t="s">
         <v>90</v>
       </c>
-      <c r="S2" s="48"/>
-      <c r="T2" s="48"/>
-      <c r="U2" s="48"/>
-      <c r="V2" s="48"/>
-      <c r="W2" s="48"/>
-    </row>
-    <row r="3" spans="2:23" ht="15">
+      <c r="S2" s="96"/>
+      <c r="T2" s="96"/>
+      <c r="U2" s="96"/>
+      <c r="V2" s="96"/>
+      <c r="W2" s="96"/>
+    </row>
+    <row r="3" spans="2:23">
       <c r="B3" s="8" t="s">
         <v>242</v>
       </c>
       <c r="Q3" s="18" t="s">
         <v>233</v>
       </c>
-      <c r="R3" s="46" t="s">
+      <c r="R3" s="94" t="s">
         <v>234</v>
       </c>
-      <c r="S3" s="46"/>
-      <c r="T3" s="46"/>
-      <c r="U3" s="46"/>
-      <c r="V3" s="46"/>
-      <c r="W3" s="46"/>
-    </row>
-    <row r="4" spans="2:23" ht="23.25">
+      <c r="S3" s="94"/>
+      <c r="T3" s="94"/>
+      <c r="U3" s="94"/>
+      <c r="V3" s="94"/>
+      <c r="W3" s="94"/>
+    </row>
+    <row r="4" spans="2:23" ht="22.8">
       <c r="B4" s="20" t="s">
         <v>223</v>
       </c>
       <c r="Q4" s="18" t="s">
         <v>235</v>
       </c>
-      <c r="R4" s="46" t="s">
+      <c r="R4" s="94" t="s">
         <v>236</v>
       </c>
-      <c r="S4" s="46"/>
-      <c r="T4" s="46"/>
-      <c r="U4" s="46"/>
-      <c r="V4" s="46"/>
-      <c r="W4" s="46"/>
-    </row>
-    <row r="5" spans="2:23" ht="15">
+      <c r="S4" s="94"/>
+      <c r="T4" s="94"/>
+      <c r="U4" s="94"/>
+      <c r="V4" s="94"/>
+      <c r="W4" s="94"/>
+    </row>
+    <row r="5" spans="2:23">
       <c r="B5" s="8" t="s">
         <v>243</v>
       </c>
       <c r="Q5" s="18" t="s">
         <v>237</v>
       </c>
-      <c r="R5" s="46" t="s">
+      <c r="R5" s="94" t="s">
         <v>238</v>
       </c>
-      <c r="S5" s="46"/>
-      <c r="T5" s="46"/>
-      <c r="U5" s="46"/>
-      <c r="V5" s="46"/>
-      <c r="W5" s="46"/>
+      <c r="S5" s="94"/>
+      <c r="T5" s="94"/>
+      <c r="U5" s="94"/>
+      <c r="V5" s="94"/>
+      <c r="W5" s="94"/>
     </row>
     <row r="6" spans="2:23">
       <c r="C6" s="21" t="s">
@@ -10369,30 +10281,30 @@
       <c r="Q6" s="18" t="s">
         <v>239</v>
       </c>
-      <c r="R6" s="46" t="s">
+      <c r="R6" s="94" t="s">
         <v>240</v>
       </c>
-      <c r="S6" s="46"/>
-      <c r="T6" s="46"/>
-      <c r="U6" s="46"/>
-      <c r="V6" s="46"/>
-      <c r="W6" s="46"/>
-    </row>
-    <row r="7" spans="2:23" ht="15">
+      <c r="S6" s="94"/>
+      <c r="T6" s="94"/>
+      <c r="U6" s="94"/>
+      <c r="V6" s="94"/>
+      <c r="W6" s="94"/>
+    </row>
+    <row r="7" spans="2:23">
       <c r="B7" s="8" t="s">
         <v>244</v>
       </c>
       <c r="Q7" s="19" t="s">
         <v>241</v>
       </c>
-      <c r="R7" s="46" t="s">
+      <c r="R7" s="94" t="s">
         <v>252</v>
       </c>
-      <c r="S7" s="46"/>
-      <c r="T7" s="46"/>
-      <c r="U7" s="46"/>
-      <c r="V7" s="46"/>
-      <c r="W7" s="46"/>
+      <c r="S7" s="94"/>
+      <c r="T7" s="94"/>
+      <c r="U7" s="94"/>
+      <c r="V7" s="94"/>
+      <c r="W7" s="94"/>
     </row>
     <row r="8" spans="2:23">
       <c r="C8" s="5" t="s">
@@ -10412,7 +10324,7 @@
       <c r="J9" s="22"/>
       <c r="K9" s="22"/>
     </row>
-    <row r="11" spans="2:23" ht="17.25">
+    <row r="11" spans="2:23" ht="17.399999999999999">
       <c r="B11" s="2" t="s">
         <v>226</v>
       </c>
@@ -10427,38 +10339,38 @@
         <v>247</v>
       </c>
     </row>
-    <row r="14" spans="2:23" ht="23.25">
+    <row r="14" spans="2:23" ht="22.8">
       <c r="B14" s="3"/>
       <c r="C14" s="20" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="16" spans="2:23" ht="17.25">
+    <row r="16" spans="2:23" ht="17.399999999999999">
       <c r="B16" s="2" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="17" spans="2:3" ht="15">
+    <row r="17" spans="2:3">
       <c r="C17" s="3" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="18" spans="2:3" ht="15">
+    <row r="18" spans="2:3">
       <c r="C18" s="8" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="19" spans="2:3" ht="15">
+    <row r="19" spans="2:3">
       <c r="C19" s="3" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="20" spans="2:3" ht="17.25">
+    <row r="20" spans="2:3" ht="17.399999999999999">
       <c r="B20" s="2" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="21" spans="2:3" ht="23.25">
+    <row r="21" spans="2:3" ht="22.8">
       <c r="C21" s="3" t="s">
         <v>253</v>
       </c>
@@ -10483,7 +10395,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="29" spans="2:3" ht="23.25">
+    <row r="29" spans="2:3" ht="22.8">
       <c r="B29" s="1"/>
     </row>
   </sheetData>
@@ -10502,9 +10414,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAF25B4A-EE7F-44E0-86AA-C29FDAAB9ED9}">
   <dimension ref="B1:L47"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <sheetData>
-    <row r="1" spans="2:6" ht="23.25">
+    <row r="1" spans="2:6" ht="22.8">
       <c r="B1" s="1" t="s">
         <v>254</v>
       </c>
@@ -10514,7 +10426,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="3" spans="2:6" ht="15">
+    <row r="3" spans="2:6">
       <c r="B3" s="8" t="s">
         <v>256</v>
       </c>
@@ -10524,17 +10436,17 @@
         <v>257</v>
       </c>
     </row>
-    <row r="5" spans="2:6" ht="23.25">
+    <row r="5" spans="2:6" ht="22.8">
       <c r="B5" s="20" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="6" spans="2:6" ht="15">
+    <row r="6" spans="2:6">
       <c r="B6" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="8" spans="2:6" ht="23.25">
+    <row r="8" spans="2:6" ht="22.8">
       <c r="B8" s="1" t="s">
         <v>260</v>
       </c>
@@ -10591,140 +10503,140 @@
       <c r="E17" s="29"/>
       <c r="F17" s="30"/>
     </row>
-    <row r="19" spans="2:12" ht="17.25">
+    <row r="19" spans="2:12" ht="17.399999999999999">
       <c r="B19" s="2" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="21" spans="2:12" ht="15">
-      <c r="C21" s="33" t="s">
+    <row r="21" spans="2:12">
+      <c r="C21" s="81" t="s">
         <v>270</v>
       </c>
-      <c r="D21" s="33"/>
-      <c r="E21" s="33"/>
-      <c r="F21" s="33" t="s">
+      <c r="D21" s="81"/>
+      <c r="E21" s="81"/>
+      <c r="F21" s="81" t="s">
         <v>186</v>
       </c>
-      <c r="G21" s="33"/>
-      <c r="H21" s="33"/>
-      <c r="I21" s="33"/>
-      <c r="J21" s="33"/>
-      <c r="K21" s="33"/>
-      <c r="L21" s="33"/>
+      <c r="G21" s="81"/>
+      <c r="H21" s="81"/>
+      <c r="I21" s="81"/>
+      <c r="J21" s="81"/>
+      <c r="K21" s="81"/>
+      <c r="L21" s="81"/>
     </row>
     <row r="22" spans="2:12">
-      <c r="C22" s="35" t="s">
+      <c r="C22" s="83" t="s">
         <v>271</v>
       </c>
-      <c r="D22" s="35"/>
-      <c r="E22" s="35"/>
-      <c r="F22" s="34" t="s">
+      <c r="D22" s="83"/>
+      <c r="E22" s="83"/>
+      <c r="F22" s="82" t="s">
         <v>272</v>
       </c>
-      <c r="G22" s="34"/>
-      <c r="H22" s="34"/>
-      <c r="I22" s="34"/>
-      <c r="J22" s="34"/>
-      <c r="K22" s="34"/>
-      <c r="L22" s="34"/>
+      <c r="G22" s="82"/>
+      <c r="H22" s="82"/>
+      <c r="I22" s="82"/>
+      <c r="J22" s="82"/>
+      <c r="K22" s="82"/>
+      <c r="L22" s="82"/>
     </row>
     <row r="23" spans="2:12">
-      <c r="C23" s="35" t="s">
+      <c r="C23" s="83" t="s">
         <v>273</v>
       </c>
-      <c r="D23" s="35"/>
-      <c r="E23" s="35"/>
-      <c r="F23" s="34" t="s">
+      <c r="D23" s="83"/>
+      <c r="E23" s="83"/>
+      <c r="F23" s="82" t="s">
         <v>274</v>
       </c>
-      <c r="G23" s="34"/>
-      <c r="H23" s="34"/>
-      <c r="I23" s="34"/>
-      <c r="J23" s="34"/>
-      <c r="K23" s="34"/>
-      <c r="L23" s="34"/>
+      <c r="G23" s="82"/>
+      <c r="H23" s="82"/>
+      <c r="I23" s="82"/>
+      <c r="J23" s="82"/>
+      <c r="K23" s="82"/>
+      <c r="L23" s="82"/>
     </row>
     <row r="24" spans="2:12">
-      <c r="C24" s="35" t="s">
+      <c r="C24" s="83" t="s">
         <v>275</v>
       </c>
-      <c r="D24" s="35"/>
-      <c r="E24" s="35"/>
-      <c r="F24" s="34" t="s">
+      <c r="D24" s="83"/>
+      <c r="E24" s="83"/>
+      <c r="F24" s="82" t="s">
         <v>276</v>
       </c>
-      <c r="G24" s="34"/>
-      <c r="H24" s="34"/>
-      <c r="I24" s="34"/>
-      <c r="J24" s="34"/>
-      <c r="K24" s="34"/>
-      <c r="L24" s="34"/>
+      <c r="G24" s="82"/>
+      <c r="H24" s="82"/>
+      <c r="I24" s="82"/>
+      <c r="J24" s="82"/>
+      <c r="K24" s="82"/>
+      <c r="L24" s="82"/>
     </row>
     <row r="25" spans="2:12">
-      <c r="C25" s="35" t="s">
+      <c r="C25" s="83" t="s">
         <v>277</v>
       </c>
-      <c r="D25" s="35"/>
-      <c r="E25" s="35"/>
-      <c r="F25" s="34" t="s">
+      <c r="D25" s="83"/>
+      <c r="E25" s="83"/>
+      <c r="F25" s="82" t="s">
         <v>278</v>
       </c>
-      <c r="G25" s="34"/>
-      <c r="H25" s="34"/>
-      <c r="I25" s="34"/>
-      <c r="J25" s="34"/>
-      <c r="K25" s="34"/>
-      <c r="L25" s="34"/>
+      <c r="G25" s="82"/>
+      <c r="H25" s="82"/>
+      <c r="I25" s="82"/>
+      <c r="J25" s="82"/>
+      <c r="K25" s="82"/>
+      <c r="L25" s="82"/>
     </row>
     <row r="26" spans="2:12">
-      <c r="C26" s="35" t="s">
+      <c r="C26" s="83" t="s">
         <v>187</v>
       </c>
-      <c r="D26" s="35"/>
-      <c r="E26" s="35"/>
-      <c r="F26" s="34" t="s">
+      <c r="D26" s="83"/>
+      <c r="E26" s="83"/>
+      <c r="F26" s="82" t="s">
         <v>279</v>
       </c>
-      <c r="G26" s="34"/>
-      <c r="H26" s="34"/>
-      <c r="I26" s="34"/>
-      <c r="J26" s="34"/>
-      <c r="K26" s="34"/>
-      <c r="L26" s="34"/>
+      <c r="G26" s="82"/>
+      <c r="H26" s="82"/>
+      <c r="I26" s="82"/>
+      <c r="J26" s="82"/>
+      <c r="K26" s="82"/>
+      <c r="L26" s="82"/>
     </row>
     <row r="27" spans="2:12">
-      <c r="C27" s="35" t="s">
+      <c r="C27" s="83" t="s">
         <v>280</v>
       </c>
-      <c r="D27" s="35"/>
-      <c r="E27" s="35"/>
-      <c r="F27" s="34" t="s">
+      <c r="D27" s="83"/>
+      <c r="E27" s="83"/>
+      <c r="F27" s="82" t="s">
         <v>281</v>
       </c>
-      <c r="G27" s="34"/>
-      <c r="H27" s="34"/>
-      <c r="I27" s="34"/>
-      <c r="J27" s="34"/>
-      <c r="K27" s="34"/>
-      <c r="L27" s="34"/>
+      <c r="G27" s="82"/>
+      <c r="H27" s="82"/>
+      <c r="I27" s="82"/>
+      <c r="J27" s="82"/>
+      <c r="K27" s="82"/>
+      <c r="L27" s="82"/>
     </row>
     <row r="28" spans="2:12">
-      <c r="C28" s="35" t="s">
+      <c r="C28" s="83" t="s">
         <v>282</v>
       </c>
-      <c r="D28" s="35"/>
-      <c r="E28" s="35"/>
-      <c r="F28" s="34" t="s">
+      <c r="D28" s="83"/>
+      <c r="E28" s="83"/>
+      <c r="F28" s="82" t="s">
         <v>283</v>
       </c>
-      <c r="G28" s="34"/>
-      <c r="H28" s="34"/>
-      <c r="I28" s="34"/>
-      <c r="J28" s="34"/>
-      <c r="K28" s="34"/>
-      <c r="L28" s="34"/>
-    </row>
-    <row r="31" spans="2:12" ht="23.25">
+      <c r="G28" s="82"/>
+      <c r="H28" s="82"/>
+      <c r="I28" s="82"/>
+      <c r="J28" s="82"/>
+      <c r="K28" s="82"/>
+      <c r="L28" s="82"/>
+    </row>
+    <row r="31" spans="2:12" ht="22.8">
       <c r="B31" s="1" t="s">
         <v>284</v>
       </c>
@@ -10739,63 +10651,63 @@
         <v>286</v>
       </c>
     </row>
-    <row r="34" spans="2:8" ht="15">
+    <row r="34" spans="2:8" ht="27.6">
       <c r="C34" s="31" t="s">
         <v>287</v>
       </c>
-      <c r="D34" s="49" t="s">
+      <c r="D34" s="97" t="s">
         <v>186</v>
       </c>
-      <c r="E34" s="49"/>
-      <c r="F34" s="49"/>
-      <c r="G34" s="49"/>
-      <c r="H34" s="49"/>
+      <c r="E34" s="97"/>
+      <c r="F34" s="97"/>
+      <c r="G34" s="97"/>
+      <c r="H34" s="97"/>
     </row>
     <row r="35" spans="2:8">
       <c r="C35" s="32" t="s">
         <v>288</v>
       </c>
-      <c r="D35" s="50" t="s">
+      <c r="D35" s="98" t="s">
         <v>289</v>
       </c>
-      <c r="E35" s="50"/>
-      <c r="F35" s="50"/>
-      <c r="G35" s="50"/>
-      <c r="H35" s="50"/>
+      <c r="E35" s="98"/>
+      <c r="F35" s="98"/>
+      <c r="G35" s="98"/>
+      <c r="H35" s="98"/>
     </row>
     <row r="36" spans="2:8">
       <c r="C36" s="32" t="s">
         <v>290</v>
       </c>
-      <c r="D36" s="50" t="s">
+      <c r="D36" s="98" t="s">
         <v>291</v>
       </c>
-      <c r="E36" s="50"/>
-      <c r="F36" s="50"/>
-      <c r="G36" s="50"/>
-      <c r="H36" s="50"/>
+      <c r="E36" s="98"/>
+      <c r="F36" s="98"/>
+      <c r="G36" s="98"/>
+      <c r="H36" s="98"/>
     </row>
     <row r="37" spans="2:8">
       <c r="C37" s="32" t="s">
         <v>292</v>
       </c>
-      <c r="D37" s="50" t="s">
+      <c r="D37" s="98" t="s">
         <v>293</v>
       </c>
-      <c r="E37" s="50"/>
-      <c r="F37" s="50"/>
-      <c r="G37" s="50"/>
-      <c r="H37" s="50"/>
+      <c r="E37" s="98"/>
+      <c r="F37" s="98"/>
+      <c r="G37" s="98"/>
+      <c r="H37" s="98"/>
     </row>
     <row r="38" spans="2:8">
       <c r="B38" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="42" spans="2:8" ht="23.25">
+    <row r="42" spans="2:8" ht="22.8">
       <c r="B42" s="1"/>
     </row>
-    <row r="44" spans="2:8" ht="15">
+    <row r="44" spans="2:8">
       <c r="B44" s="6"/>
       <c r="C44" s="6"/>
     </row>
@@ -10841,20 +10753,20 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A4EAA29-30A3-461D-98E6-BDBCFC321088}">
   <dimension ref="B1:D68"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <sheetData>
-    <row r="1" spans="2:4" ht="23.25">
+    <row r="1" spans="2:4" ht="22.8">
       <c r="B1" s="1" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="2" spans="2:4" ht="15">
+    <row r="2" spans="2:4">
       <c r="C2" t="s">
         <v>300</v>
       </c>
     </row>
     <row r="3" spans="2:4">
-      <c r="C3" s="52" t="s">
+      <c r="C3" s="34" t="s">
         <v>301</v>
       </c>
     </row>
@@ -10868,7 +10780,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="23.25">
+    <row r="6" spans="2:4" ht="22.8">
       <c r="B6" s="1" t="s">
         <v>304</v>
       </c>
@@ -10903,8 +10815,8 @@
         <v>295</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="15">
-      <c r="C14" s="54" t="s">
+    <row r="14" spans="2:4">
+      <c r="C14" s="36" t="s">
         <v>336</v>
       </c>
     </row>
@@ -10923,7 +10835,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="18" spans="2:4" ht="23.25">
+    <row r="18" spans="2:4" ht="22.8">
       <c r="B18" s="1" t="s">
         <v>312</v>
       </c>
@@ -10933,22 +10845,22 @@
         <v>313</v>
       </c>
     </row>
-    <row r="20" spans="2:4" ht="15">
+    <row r="20" spans="2:4">
       <c r="C20" t="s">
         <v>314</v>
       </c>
     </row>
     <row r="21" spans="2:4">
-      <c r="C21" s="52" t="s">
+      <c r="C21" s="34" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="22" spans="2:4" ht="23.25">
+    <row r="22" spans="2:4" ht="22.8">
       <c r="B22" s="1" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="23" spans="2:4" ht="17.25">
+    <row r="23" spans="2:4" ht="17.399999999999999">
       <c r="C23" s="2" t="s">
         <v>317</v>
       </c>
@@ -10978,7 +10890,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="30" spans="2:4" ht="17.25">
+    <row r="30" spans="2:4" ht="17.399999999999999">
       <c r="C30" s="2" t="s">
         <v>322</v>
       </c>
@@ -11063,58 +10975,58 @@
         <v>298</v>
       </c>
     </row>
-    <row r="51" spans="2:3" ht="23.25">
+    <row r="51" spans="2:3" ht="22.8">
       <c r="B51" s="1"/>
     </row>
-    <row r="53" spans="2:3" ht="15">
+    <row r="53" spans="2:3">
       <c r="B53" s="6"/>
       <c r="C53" s="6"/>
     </row>
     <row r="54" spans="2:3">
-      <c r="B54" s="53"/>
-      <c r="C54" s="53"/>
+      <c r="B54" s="35"/>
+      <c r="C54" s="35"/>
     </row>
     <row r="55" spans="2:3">
-      <c r="B55" s="53"/>
-      <c r="C55" s="53"/>
+      <c r="B55" s="35"/>
+      <c r="C55" s="35"/>
     </row>
     <row r="56" spans="2:3">
       <c r="B56" s="7"/>
       <c r="C56" s="7"/>
     </row>
     <row r="57" spans="2:3">
-      <c r="B57" s="53"/>
-      <c r="C57" s="53"/>
+      <c r="B57" s="35"/>
+      <c r="C57" s="35"/>
     </row>
     <row r="58" spans="2:3">
       <c r="B58" s="7"/>
       <c r="C58" s="7"/>
     </row>
-    <row r="61" spans="2:3" ht="23.25">
+    <row r="61" spans="2:3" ht="22.8">
       <c r="B61" s="1"/>
     </row>
-    <row r="63" spans="2:3" ht="15">
+    <row r="63" spans="2:3">
       <c r="B63" s="6"/>
       <c r="C63" s="6"/>
     </row>
     <row r="64" spans="2:3">
-      <c r="B64" s="53"/>
+      <c r="B64" s="35"/>
       <c r="C64" s="7"/>
     </row>
     <row r="65" spans="2:3">
-      <c r="B65" s="53"/>
+      <c r="B65" s="35"/>
       <c r="C65" s="7"/>
     </row>
     <row r="66" spans="2:3">
-      <c r="B66" s="53"/>
+      <c r="B66" s="35"/>
       <c r="C66" s="7"/>
     </row>
     <row r="67" spans="2:3">
-      <c r="B67" s="53"/>
+      <c r="B67" s="35"/>
       <c r="C67" s="7"/>
     </row>
     <row r="68" spans="2:3">
-      <c r="B68" s="53"/>
+      <c r="B68" s="35"/>
       <c r="C68" s="7"/>
     </row>
   </sheetData>

</xml_diff>